<commit_message>
finalized peak picking, reordered figure numbers
</commit_message>
<xml_diff>
--- a/results/pp_human/Additional Human Picked Peaks [v3, scipy, prom_C=3, prom_mag=2, hpf_meth=HPF=(300Hz cf, 50Hz df, 100dB rip), fs=44100, tau=69.66ms, xi=15.08ms, hop_C=hop_mag=10.0ms, rho=1.0, hann, win_mag=hann, avg_meth=power, flim=[500, inf], wf_len_s=None].xlsx
+++ b/results/pp_human/Additional Human Picked Peaks [v3, scipy, prom_C=3, prom_mag=2, hpf_meth=HPF=(300Hz cf, 50Hz df, 100dB rip), fs=44100, tau=69.66ms, xi=15.08ms, hop_C=hop_mag=10.0ms, rho=1.0, hann, win_mag=hann, avg_meth=power, flim=[500, inf], wf_len_s=None].xlsx
@@ -1958,7 +1958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L216"/>
+  <dimension ref="A1:L198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2602,7 +2602,7 @@
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="n">
-        <v>4450.1953125</v>
+        <v>6574.8046875</v>
       </c>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
@@ -2617,10 +2617,10 @@
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
-      <c r="B39" t="n">
-        <v>6574.8046875</v>
-      </c>
-      <c r="C39" t="inlineStr"/>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="n">
+        <v>617.28515625</v>
+      </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr"/>
@@ -2635,7 +2635,7 @@
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="n">
-        <v>617.28515625</v>
+        <v>732.12890625</v>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr"/>
@@ -2651,7 +2651,7 @@
       <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="n">
-        <v>732.12890625</v>
+        <v>803.90625</v>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr"/>
@@ -2667,7 +2667,7 @@
       <c r="A42" t="inlineStr"/>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="n">
-        <v>803.90625</v>
+        <v>918.75</v>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr"/>
@@ -2683,7 +2683,7 @@
       <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="n">
-        <v>918.75</v>
+        <v>990.52734375</v>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr"/>
@@ -2699,7 +2699,7 @@
       <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="n">
-        <v>990.52734375</v>
+        <v>1076.66015625</v>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr"/>
@@ -2715,7 +2715,7 @@
       <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="n">
-        <v>1076.66015625</v>
+        <v>1134.08203125</v>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr"/>
@@ -2731,7 +2731,7 @@
       <c r="A46" t="inlineStr"/>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="n">
-        <v>1134.08203125</v>
+        <v>1263.28125</v>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr"/>
@@ -2747,7 +2747,7 @@
       <c r="A47" t="inlineStr"/>
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="n">
-        <v>1263.28125</v>
+        <v>1320.703125</v>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr"/>
@@ -2763,7 +2763,7 @@
       <c r="A48" t="inlineStr"/>
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="n">
-        <v>1320.703125</v>
+        <v>1449.90234375</v>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr"/>
@@ -2779,7 +2779,7 @@
       <c r="A49" t="inlineStr"/>
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="n">
-        <v>1449.90234375</v>
+        <v>1507.32421875</v>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr"/>
@@ -2795,7 +2795,7 @@
       <c r="A50" t="inlineStr"/>
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="n">
-        <v>1507.32421875</v>
+        <v>1579.1015625</v>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr"/>
@@ -2811,7 +2811,7 @@
       <c r="A51" t="inlineStr"/>
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="n">
-        <v>1579.1015625</v>
+        <v>1665.234375</v>
       </c>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr"/>
@@ -2827,7 +2827,7 @@
       <c r="A52" t="inlineStr"/>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="n">
-        <v>1665.234375</v>
+        <v>1737.01171875</v>
       </c>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr"/>
@@ -2843,7 +2843,7 @@
       <c r="A53" t="inlineStr"/>
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="n">
-        <v>1737.01171875</v>
+        <v>1794.43359375</v>
       </c>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr"/>
@@ -2859,7 +2859,7 @@
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="n">
-        <v>1794.43359375</v>
+        <v>2268.1640625</v>
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr"/>
@@ -2875,7 +2875,7 @@
       <c r="A55" t="inlineStr"/>
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="n">
-        <v>2268.1640625</v>
+        <v>3646.2890625</v>
       </c>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr"/>
@@ -2891,7 +2891,7 @@
       <c r="A56" t="inlineStr"/>
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="n">
-        <v>3646.2890625</v>
+        <v>3861.62109375</v>
       </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr"/>
@@ -2907,7 +2907,7 @@
       <c r="A57" t="inlineStr"/>
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="n">
-        <v>3861.62109375</v>
+        <v>4019.53125</v>
       </c>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr"/>
@@ -2923,7 +2923,7 @@
       <c r="A58" t="inlineStr"/>
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="n">
-        <v>4019.53125</v>
+        <v>4177.44140625</v>
       </c>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr"/>
@@ -2939,7 +2939,7 @@
       <c r="A59" t="inlineStr"/>
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="n">
-        <v>4177.44140625</v>
+        <v>4694.23828125</v>
       </c>
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr"/>
@@ -2955,7 +2955,7 @@
       <c r="A60" t="inlineStr"/>
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="n">
-        <v>4694.23828125</v>
+        <v>5656.0546875</v>
       </c>
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr"/>
@@ -2971,7 +2971,7 @@
       <c r="A61" t="inlineStr"/>
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="n">
-        <v>5656.0546875</v>
+        <v>6761.42578125</v>
       </c>
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr"/>
@@ -2987,7 +2987,7 @@
       <c r="A62" t="inlineStr"/>
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="n">
-        <v>6761.42578125</v>
+        <v>7048.53515625</v>
       </c>
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr"/>
@@ -3003,7 +3003,7 @@
       <c r="A63" t="inlineStr"/>
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="n">
-        <v>7048.53515625</v>
+        <v>7335.64453125</v>
       </c>
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr"/>
@@ -3019,7 +3019,7 @@
       <c r="A64" t="inlineStr"/>
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="n">
-        <v>7335.64453125</v>
+        <v>7622.75390625</v>
       </c>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr"/>
@@ -3035,7 +3035,7 @@
       <c r="A65" t="inlineStr"/>
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="n">
-        <v>7622.75390625</v>
+        <v>9072.65625</v>
       </c>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr"/>
@@ -3050,10 +3050,10 @@
     <row r="66">
       <c r="A66" t="inlineStr"/>
       <c r="B66" t="inlineStr"/>
-      <c r="C66" t="n">
-        <v>9072.65625</v>
-      </c>
-      <c r="D66" t="inlineStr"/>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="n">
+        <v>645.99609375</v>
+      </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr"/>
@@ -3068,7 +3068,7 @@
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr"/>
       <c r="D67" t="n">
-        <v>645.99609375</v>
+        <v>746.484375</v>
       </c>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr"/>
@@ -3084,7 +3084,7 @@
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="n">
-        <v>746.484375</v>
+        <v>861.328125</v>
       </c>
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr"/>
@@ -3100,7 +3100,7 @@
       <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr"/>
       <c r="D69" t="n">
-        <v>861.328125</v>
+        <v>990.52734375</v>
       </c>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr"/>
@@ -3116,7 +3116,7 @@
       <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr"/>
       <c r="D70" t="n">
-        <v>990.52734375</v>
+        <v>1047.94921875</v>
       </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
@@ -3132,7 +3132,7 @@
       <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr"/>
       <c r="D71" t="n">
-        <v>1047.94921875</v>
+        <v>1306.34765625</v>
       </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr"/>
@@ -3148,7 +3148,7 @@
       <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr"/>
       <c r="D72" t="n">
-        <v>1306.34765625</v>
+        <v>1478.61328125</v>
       </c>
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr"/>
@@ -3164,7 +3164,7 @@
       <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr"/>
       <c r="D73" t="n">
-        <v>1478.61328125</v>
+        <v>1550.390625</v>
       </c>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr"/>
@@ -3180,7 +3180,7 @@
       <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr"/>
       <c r="D74" t="n">
-        <v>1550.390625</v>
+        <v>1622.16796875</v>
       </c>
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr"/>
@@ -3196,7 +3196,7 @@
       <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr"/>
       <c r="D75" t="n">
-        <v>1622.16796875</v>
+        <v>1722.65625</v>
       </c>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr"/>
@@ -3212,7 +3212,7 @@
       <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr"/>
       <c r="D76" t="n">
-        <v>1722.65625</v>
+        <v>1794.43359375</v>
       </c>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr"/>
@@ -3228,7 +3228,7 @@
       <c r="B77" t="inlineStr"/>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="n">
-        <v>1794.43359375</v>
+        <v>1894.921875</v>
       </c>
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr"/>
@@ -3244,7 +3244,7 @@
       <c r="B78" t="inlineStr"/>
       <c r="C78" t="inlineStr"/>
       <c r="D78" t="n">
-        <v>1894.921875</v>
+        <v>2024.12109375</v>
       </c>
       <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr"/>
@@ -3260,7 +3260,7 @@
       <c r="B79" t="inlineStr"/>
       <c r="C79" t="inlineStr"/>
       <c r="D79" t="n">
-        <v>2024.12109375</v>
+        <v>2239.453125</v>
       </c>
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr"/>
@@ -3276,7 +3276,7 @@
       <c r="B80" t="inlineStr"/>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>2124.609375</v>
+        <v>2756.25</v>
       </c>
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr"/>
@@ -3292,7 +3292,7 @@
       <c r="B81" t="inlineStr"/>
       <c r="C81" t="inlineStr"/>
       <c r="D81" t="n">
-        <v>2239.453125</v>
+        <v>3043.359375</v>
       </c>
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr"/>
@@ -3308,7 +3308,7 @@
       <c r="B82" t="inlineStr"/>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="n">
-        <v>2756.25</v>
+        <v>3172.55859375</v>
       </c>
       <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr"/>
@@ -3324,7 +3324,7 @@
       <c r="B83" t="inlineStr"/>
       <c r="C83" t="inlineStr"/>
       <c r="D83" t="n">
-        <v>3043.359375</v>
+        <v>4005.17578125</v>
       </c>
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr"/>
@@ -3340,7 +3340,7 @@
       <c r="B84" t="inlineStr"/>
       <c r="C84" t="inlineStr"/>
       <c r="D84" t="n">
-        <v>3172.55859375</v>
+        <v>4177.44140625</v>
       </c>
       <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr"/>
@@ -3355,10 +3355,10 @@
       <c r="A85" t="inlineStr"/>
       <c r="B85" t="inlineStr"/>
       <c r="C85" t="inlineStr"/>
-      <c r="D85" t="n">
-        <v>4005.17578125</v>
-      </c>
-      <c r="E85" t="inlineStr"/>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="n">
+        <v>602.9296875</v>
+      </c>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr"/>
@@ -3371,10 +3371,10 @@
       <c r="A86" t="inlineStr"/>
       <c r="B86" t="inlineStr"/>
       <c r="C86" t="inlineStr"/>
-      <c r="D86" t="n">
-        <v>4177.44140625</v>
-      </c>
-      <c r="E86" t="inlineStr"/>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="n">
+        <v>732.12890625</v>
+      </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr"/>
@@ -3389,7 +3389,7 @@
       <c r="C87" t="inlineStr"/>
       <c r="D87" t="inlineStr"/>
       <c r="E87" t="n">
-        <v>602.9296875</v>
+        <v>789.55078125</v>
       </c>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr"/>
@@ -3405,7 +3405,7 @@
       <c r="C88" t="inlineStr"/>
       <c r="D88" t="inlineStr"/>
       <c r="E88" t="n">
-        <v>732.12890625</v>
+        <v>846.97265625</v>
       </c>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr"/>
@@ -3421,7 +3421,7 @@
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="inlineStr"/>
       <c r="E89" t="n">
-        <v>789.55078125</v>
+        <v>904.39453125</v>
       </c>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
@@ -3437,7 +3437,7 @@
       <c r="C90" t="inlineStr"/>
       <c r="D90" t="inlineStr"/>
       <c r="E90" t="n">
-        <v>846.97265625</v>
+        <v>1234.5703125</v>
       </c>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr"/>
@@ -3453,7 +3453,7 @@
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="inlineStr"/>
       <c r="E91" t="n">
-        <v>904.39453125</v>
+        <v>1435.546875</v>
       </c>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr"/>
@@ -3469,7 +3469,7 @@
       <c r="C92" t="inlineStr"/>
       <c r="D92" t="inlineStr"/>
       <c r="E92" t="n">
-        <v>1119.7265625</v>
+        <v>1708.30078125</v>
       </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
@@ -3485,7 +3485,7 @@
       <c r="C93" t="inlineStr"/>
       <c r="D93" t="inlineStr"/>
       <c r="E93" t="n">
-        <v>1234.5703125</v>
+        <v>1966.69921875</v>
       </c>
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr"/>
@@ -3501,7 +3501,7 @@
       <c r="C94" t="inlineStr"/>
       <c r="D94" t="inlineStr"/>
       <c r="E94" t="n">
-        <v>1435.546875</v>
+        <v>3560.15625</v>
       </c>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr"/>
@@ -3517,7 +3517,7 @@
       <c r="C95" t="inlineStr"/>
       <c r="D95" t="inlineStr"/>
       <c r="E95" t="n">
-        <v>1708.30078125</v>
+        <v>4062.59765625</v>
       </c>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
@@ -3533,7 +3533,7 @@
       <c r="C96" t="inlineStr"/>
       <c r="D96" t="inlineStr"/>
       <c r="E96" t="n">
-        <v>1966.69921875</v>
+        <v>4981.34765625</v>
       </c>
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr"/>
@@ -3549,7 +3549,7 @@
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="inlineStr"/>
       <c r="E97" t="n">
-        <v>2942.87109375</v>
+        <v>7278.22265625</v>
       </c>
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr"/>
@@ -3564,10 +3564,10 @@
       <c r="B98" t="inlineStr"/>
       <c r="C98" t="inlineStr"/>
       <c r="D98" t="inlineStr"/>
-      <c r="E98" t="n">
-        <v>3560.15625</v>
-      </c>
-      <c r="F98" t="inlineStr"/>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="n">
+        <v>1076.66015625</v>
+      </c>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr"/>
       <c r="I98" t="inlineStr"/>
@@ -3580,10 +3580,10 @@
       <c r="B99" t="inlineStr"/>
       <c r="C99" t="inlineStr"/>
       <c r="D99" t="inlineStr"/>
-      <c r="E99" t="n">
-        <v>3861.62109375</v>
-      </c>
-      <c r="F99" t="inlineStr"/>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="n">
+        <v>1119.7265625</v>
+      </c>
       <c r="G99" t="inlineStr"/>
       <c r="H99" t="inlineStr"/>
       <c r="I99" t="inlineStr"/>
@@ -3596,10 +3596,10 @@
       <c r="B100" t="inlineStr"/>
       <c r="C100" t="inlineStr"/>
       <c r="D100" t="inlineStr"/>
-      <c r="E100" t="n">
-        <v>4062.59765625</v>
-      </c>
-      <c r="F100" t="inlineStr"/>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="n">
+        <v>1291.9921875</v>
+      </c>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr"/>
       <c r="I100" t="inlineStr"/>
@@ -3612,10 +3612,10 @@
       <c r="B101" t="inlineStr"/>
       <c r="C101" t="inlineStr"/>
       <c r="D101" t="inlineStr"/>
-      <c r="E101" t="n">
-        <v>4378.41796875</v>
-      </c>
-      <c r="F101" t="inlineStr"/>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="n">
+        <v>1579.1015625</v>
+      </c>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="inlineStr"/>
       <c r="I101" t="inlineStr"/>
@@ -3628,10 +3628,10 @@
       <c r="B102" t="inlineStr"/>
       <c r="C102" t="inlineStr"/>
       <c r="D102" t="inlineStr"/>
-      <c r="E102" t="n">
-        <v>4981.34765625</v>
-      </c>
-      <c r="F102" t="inlineStr"/>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="n">
+        <v>1722.65625</v>
+      </c>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="inlineStr"/>
       <c r="I102" t="inlineStr"/>
@@ -3644,10 +3644,10 @@
       <c r="B103" t="inlineStr"/>
       <c r="C103" t="inlineStr"/>
       <c r="D103" t="inlineStr"/>
-      <c r="E103" t="n">
-        <v>7278.22265625</v>
-      </c>
-      <c r="F103" t="inlineStr"/>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="n">
+        <v>1837.5</v>
+      </c>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr"/>
       <c r="I103" t="inlineStr"/>
@@ -3662,7 +3662,7 @@
       <c r="D104" t="inlineStr"/>
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="n">
-        <v>1076.66015625</v>
+        <v>2339.94140625</v>
       </c>
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="inlineStr"/>
@@ -3678,7 +3678,7 @@
       <c r="D105" t="inlineStr"/>
       <c r="E105" t="inlineStr"/>
       <c r="F105" t="n">
-        <v>1119.7265625</v>
+        <v>2813.671875</v>
       </c>
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="inlineStr"/>
@@ -3694,7 +3694,7 @@
       <c r="D106" t="inlineStr"/>
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="n">
-        <v>1291.9921875</v>
+        <v>3072.0703125</v>
       </c>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="inlineStr"/>
@@ -3710,7 +3710,7 @@
       <c r="D107" t="inlineStr"/>
       <c r="E107" t="inlineStr"/>
       <c r="F107" t="n">
-        <v>1579.1015625</v>
+        <v>3402.24609375</v>
       </c>
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr"/>
@@ -3726,7 +3726,7 @@
       <c r="D108" t="inlineStr"/>
       <c r="E108" t="inlineStr"/>
       <c r="F108" t="n">
-        <v>1722.65625</v>
+        <v>4048.2421875</v>
       </c>
       <c r="G108" t="inlineStr"/>
       <c r="H108" t="inlineStr"/>
@@ -3742,7 +3742,7 @@
       <c r="D109" t="inlineStr"/>
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="n">
-        <v>1837.5</v>
+        <v>5124.90234375</v>
       </c>
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr"/>
@@ -3758,7 +3758,7 @@
       <c r="D110" t="inlineStr"/>
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="n">
-        <v>2339.94140625</v>
+        <v>5842.67578125</v>
       </c>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr"/>
@@ -3774,7 +3774,7 @@
       <c r="D111" t="inlineStr"/>
       <c r="E111" t="inlineStr"/>
       <c r="F111" t="n">
-        <v>2813.671875</v>
+        <v>7938.57421875</v>
       </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr"/>
@@ -3790,7 +3790,7 @@
       <c r="D112" t="inlineStr"/>
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="n">
-        <v>3072.0703125</v>
+        <v>8311.81640625</v>
       </c>
       <c r="G112" t="inlineStr"/>
       <c r="H112" t="inlineStr"/>
@@ -3806,7 +3806,7 @@
       <c r="D113" t="inlineStr"/>
       <c r="E113" t="inlineStr"/>
       <c r="F113" t="n">
-        <v>3402.24609375</v>
+        <v>8670.703125</v>
       </c>
       <c r="G113" t="inlineStr"/>
       <c r="H113" t="inlineStr"/>
@@ -3821,10 +3821,10 @@
       <c r="C114" t="inlineStr"/>
       <c r="D114" t="inlineStr"/>
       <c r="E114" t="inlineStr"/>
-      <c r="F114" t="n">
-        <v>4048.2421875</v>
-      </c>
-      <c r="G114" t="inlineStr"/>
+      <c r="F114" t="inlineStr"/>
+      <c r="G114" t="n">
+        <v>545.5078125</v>
+      </c>
       <c r="H114" t="inlineStr"/>
       <c r="I114" t="inlineStr"/>
       <c r="J114" t="inlineStr"/>
@@ -3837,10 +3837,10 @@
       <c r="C115" t="inlineStr"/>
       <c r="D115" t="inlineStr"/>
       <c r="E115" t="inlineStr"/>
-      <c r="F115" t="n">
-        <v>5124.90234375</v>
-      </c>
-      <c r="G115" t="inlineStr"/>
+      <c r="F115" t="inlineStr"/>
+      <c r="G115" t="n">
+        <v>875.68359375</v>
+      </c>
       <c r="H115" t="inlineStr"/>
       <c r="I115" t="inlineStr"/>
       <c r="J115" t="inlineStr"/>
@@ -3853,10 +3853,10 @@
       <c r="C116" t="inlineStr"/>
       <c r="D116" t="inlineStr"/>
       <c r="E116" t="inlineStr"/>
-      <c r="F116" t="n">
-        <v>5842.67578125</v>
-      </c>
-      <c r="G116" t="inlineStr"/>
+      <c r="F116" t="inlineStr"/>
+      <c r="G116" t="n">
+        <v>1220.21484375</v>
+      </c>
       <c r="H116" t="inlineStr"/>
       <c r="I116" t="inlineStr"/>
       <c r="J116" t="inlineStr"/>
@@ -3869,10 +3869,10 @@
       <c r="C117" t="inlineStr"/>
       <c r="D117" t="inlineStr"/>
       <c r="E117" t="inlineStr"/>
-      <c r="F117" t="n">
-        <v>7938.57421875</v>
-      </c>
-      <c r="G117" t="inlineStr"/>
+      <c r="F117" t="inlineStr"/>
+      <c r="G117" t="n">
+        <v>1291.9921875</v>
+      </c>
       <c r="H117" t="inlineStr"/>
       <c r="I117" t="inlineStr"/>
       <c r="J117" t="inlineStr"/>
@@ -3885,10 +3885,10 @@
       <c r="C118" t="inlineStr"/>
       <c r="D118" t="inlineStr"/>
       <c r="E118" t="inlineStr"/>
-      <c r="F118" t="n">
-        <v>8311.81640625</v>
-      </c>
-      <c r="G118" t="inlineStr"/>
+      <c r="F118" t="inlineStr"/>
+      <c r="G118" t="n">
+        <v>1349.4140625</v>
+      </c>
       <c r="H118" t="inlineStr"/>
       <c r="I118" t="inlineStr"/>
       <c r="J118" t="inlineStr"/>
@@ -3901,10 +3901,10 @@
       <c r="C119" t="inlineStr"/>
       <c r="D119" t="inlineStr"/>
       <c r="E119" t="inlineStr"/>
-      <c r="F119" t="n">
-        <v>8670.703125</v>
-      </c>
-      <c r="G119" t="inlineStr"/>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="n">
+        <v>1492.96875</v>
+      </c>
       <c r="H119" t="inlineStr"/>
       <c r="I119" t="inlineStr"/>
       <c r="J119" t="inlineStr"/>
@@ -3919,7 +3919,7 @@
       <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="n">
-        <v>545.5078125</v>
+        <v>1880.56640625</v>
       </c>
       <c r="H120" t="inlineStr"/>
       <c r="I120" t="inlineStr"/>
@@ -3935,7 +3935,7 @@
       <c r="E121" t="inlineStr"/>
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="n">
-        <v>875.68359375</v>
+        <v>3043.359375</v>
       </c>
       <c r="H121" t="inlineStr"/>
       <c r="I121" t="inlineStr"/>
@@ -3951,7 +3951,7 @@
       <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="n">
-        <v>1105.37109375</v>
+        <v>3158.203125</v>
       </c>
       <c r="H122" t="inlineStr"/>
       <c r="I122" t="inlineStr"/>
@@ -3967,7 +3967,7 @@
       <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="n">
-        <v>1220.21484375</v>
+        <v>3301.7578125</v>
       </c>
       <c r="H123" t="inlineStr"/>
       <c r="I123" t="inlineStr"/>
@@ -3983,7 +3983,7 @@
       <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="n">
-        <v>1291.9921875</v>
+        <v>3789.84375</v>
       </c>
       <c r="H124" t="inlineStr"/>
       <c r="I124" t="inlineStr"/>
@@ -3998,10 +3998,10 @@
       <c r="D125" t="inlineStr"/>
       <c r="E125" t="inlineStr"/>
       <c r="F125" t="inlineStr"/>
-      <c r="G125" t="n">
-        <v>1349.4140625</v>
-      </c>
-      <c r="H125" t="inlineStr"/>
+      <c r="G125" t="inlineStr"/>
+      <c r="H125" t="n">
+        <v>732.12890625</v>
+      </c>
       <c r="I125" t="inlineStr"/>
       <c r="J125" t="inlineStr"/>
       <c r="K125" t="inlineStr"/>
@@ -4014,10 +4014,10 @@
       <c r="D126" t="inlineStr"/>
       <c r="E126" t="inlineStr"/>
       <c r="F126" t="inlineStr"/>
-      <c r="G126" t="n">
-        <v>1492.96875</v>
-      </c>
-      <c r="H126" t="inlineStr"/>
+      <c r="G126" t="inlineStr"/>
+      <c r="H126" t="n">
+        <v>990.52734375</v>
+      </c>
       <c r="I126" t="inlineStr"/>
       <c r="J126" t="inlineStr"/>
       <c r="K126" t="inlineStr"/>
@@ -4030,10 +4030,10 @@
       <c r="D127" t="inlineStr"/>
       <c r="E127" t="inlineStr"/>
       <c r="F127" t="inlineStr"/>
-      <c r="G127" t="n">
-        <v>1880.56640625</v>
-      </c>
-      <c r="H127" t="inlineStr"/>
+      <c r="G127" t="inlineStr"/>
+      <c r="H127" t="n">
+        <v>1205.859375</v>
+      </c>
       <c r="I127" t="inlineStr"/>
       <c r="J127" t="inlineStr"/>
       <c r="K127" t="inlineStr"/>
@@ -4046,10 +4046,10 @@
       <c r="D128" t="inlineStr"/>
       <c r="E128" t="inlineStr"/>
       <c r="F128" t="inlineStr"/>
-      <c r="G128" t="n">
-        <v>3043.359375</v>
-      </c>
-      <c r="H128" t="inlineStr"/>
+      <c r="G128" t="inlineStr"/>
+      <c r="H128" t="n">
+        <v>1291.9921875</v>
+      </c>
       <c r="I128" t="inlineStr"/>
       <c r="J128" t="inlineStr"/>
       <c r="K128" t="inlineStr"/>
@@ -4062,10 +4062,10 @@
       <c r="D129" t="inlineStr"/>
       <c r="E129" t="inlineStr"/>
       <c r="F129" t="inlineStr"/>
-      <c r="G129" t="n">
-        <v>3158.203125</v>
-      </c>
-      <c r="H129" t="inlineStr"/>
+      <c r="G129" t="inlineStr"/>
+      <c r="H129" t="n">
+        <v>1636.5234375</v>
+      </c>
       <c r="I129" t="inlineStr"/>
       <c r="J129" t="inlineStr"/>
       <c r="K129" t="inlineStr"/>
@@ -4078,10 +4078,10 @@
       <c r="D130" t="inlineStr"/>
       <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr"/>
-      <c r="G130" t="n">
-        <v>3301.7578125</v>
-      </c>
-      <c r="H130" t="inlineStr"/>
+      <c r="G130" t="inlineStr"/>
+      <c r="H130" t="n">
+        <v>2110.25390625</v>
+      </c>
       <c r="I130" t="inlineStr"/>
       <c r="J130" t="inlineStr"/>
       <c r="K130" t="inlineStr"/>
@@ -4094,10 +4094,10 @@
       <c r="D131" t="inlineStr"/>
       <c r="E131" t="inlineStr"/>
       <c r="F131" t="inlineStr"/>
-      <c r="G131" t="n">
-        <v>3789.84375</v>
-      </c>
-      <c r="H131" t="inlineStr"/>
+      <c r="G131" t="inlineStr"/>
+      <c r="H131" t="n">
+        <v>2225.09765625</v>
+      </c>
       <c r="I131" t="inlineStr"/>
       <c r="J131" t="inlineStr"/>
       <c r="K131" t="inlineStr"/>
@@ -4112,7 +4112,7 @@
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr"/>
       <c r="H132" t="n">
-        <v>645.99609375</v>
+        <v>3115.13671875</v>
       </c>
       <c r="I132" t="inlineStr"/>
       <c r="J132" t="inlineStr"/>
@@ -4128,7 +4128,7 @@
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="n">
-        <v>732.12890625</v>
+        <v>4335.3515625</v>
       </c>
       <c r="I133" t="inlineStr"/>
       <c r="J133" t="inlineStr"/>
@@ -4144,7 +4144,7 @@
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="n">
-        <v>990.52734375</v>
+        <v>5010.05859375</v>
       </c>
       <c r="I134" t="inlineStr"/>
       <c r="J134" t="inlineStr"/>
@@ -4159,10 +4159,10 @@
       <c r="E135" t="inlineStr"/>
       <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr"/>
-      <c r="H135" t="n">
-        <v>1205.859375</v>
-      </c>
-      <c r="I135" t="inlineStr"/>
+      <c r="H135" t="inlineStr"/>
+      <c r="I135" t="n">
+        <v>703.41796875</v>
+      </c>
       <c r="J135" t="inlineStr"/>
       <c r="K135" t="inlineStr"/>
       <c r="L135" t="inlineStr"/>
@@ -4175,10 +4175,10 @@
       <c r="E136" t="inlineStr"/>
       <c r="F136" t="inlineStr"/>
       <c r="G136" t="inlineStr"/>
-      <c r="H136" t="n">
-        <v>1291.9921875</v>
-      </c>
-      <c r="I136" t="inlineStr"/>
+      <c r="H136" t="inlineStr"/>
+      <c r="I136" t="n">
+        <v>990.52734375</v>
+      </c>
       <c r="J136" t="inlineStr"/>
       <c r="K136" t="inlineStr"/>
       <c r="L136" t="inlineStr"/>
@@ -4191,10 +4191,10 @@
       <c r="E137" t="inlineStr"/>
       <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr"/>
-      <c r="H137" t="n">
-        <v>1579.1015625</v>
-      </c>
-      <c r="I137" t="inlineStr"/>
+      <c r="H137" t="inlineStr"/>
+      <c r="I137" t="n">
+        <v>1679.58984375</v>
+      </c>
       <c r="J137" t="inlineStr"/>
       <c r="K137" t="inlineStr"/>
       <c r="L137" t="inlineStr"/>
@@ -4207,10 +4207,10 @@
       <c r="E138" t="inlineStr"/>
       <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr"/>
-      <c r="H138" t="n">
-        <v>1636.5234375</v>
-      </c>
-      <c r="I138" t="inlineStr"/>
+      <c r="H138" t="inlineStr"/>
+      <c r="I138" t="n">
+        <v>1780.078125</v>
+      </c>
       <c r="J138" t="inlineStr"/>
       <c r="K138" t="inlineStr"/>
       <c r="L138" t="inlineStr"/>
@@ -4223,10 +4223,10 @@
       <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr"/>
-      <c r="H139" t="n">
-        <v>2110.25390625</v>
-      </c>
-      <c r="I139" t="inlineStr"/>
+      <c r="H139" t="inlineStr"/>
+      <c r="I139" t="n">
+        <v>1894.921875</v>
+      </c>
       <c r="J139" t="inlineStr"/>
       <c r="K139" t="inlineStr"/>
       <c r="L139" t="inlineStr"/>
@@ -4239,10 +4239,10 @@
       <c r="E140" t="inlineStr"/>
       <c r="F140" t="inlineStr"/>
       <c r="G140" t="inlineStr"/>
-      <c r="H140" t="n">
-        <v>2225.09765625</v>
-      </c>
-      <c r="I140" t="inlineStr"/>
+      <c r="H140" t="inlineStr"/>
+      <c r="I140" t="n">
+        <v>2138.96484375</v>
+      </c>
       <c r="J140" t="inlineStr"/>
       <c r="K140" t="inlineStr"/>
       <c r="L140" t="inlineStr"/>
@@ -4255,10 +4255,10 @@
       <c r="E141" t="inlineStr"/>
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr"/>
-      <c r="H141" t="n">
-        <v>3115.13671875</v>
-      </c>
-      <c r="I141" t="inlineStr"/>
+      <c r="H141" t="inlineStr"/>
+      <c r="I141" t="n">
+        <v>3258.69140625</v>
+      </c>
       <c r="J141" t="inlineStr"/>
       <c r="K141" t="inlineStr"/>
       <c r="L141" t="inlineStr"/>
@@ -4271,10 +4271,10 @@
       <c r="E142" t="inlineStr"/>
       <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr"/>
-      <c r="H142" t="n">
-        <v>4335.3515625</v>
-      </c>
-      <c r="I142" t="inlineStr"/>
+      <c r="H142" t="inlineStr"/>
+      <c r="I142" t="n">
+        <v>3732.421875</v>
+      </c>
       <c r="J142" t="inlineStr"/>
       <c r="K142" t="inlineStr"/>
       <c r="L142" t="inlineStr"/>
@@ -4287,10 +4287,10 @@
       <c r="E143" t="inlineStr"/>
       <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr"/>
-      <c r="H143" t="n">
-        <v>5010.05859375</v>
-      </c>
-      <c r="I143" t="inlineStr"/>
+      <c r="H143" t="inlineStr"/>
+      <c r="I143" t="n">
+        <v>4163.0859375</v>
+      </c>
       <c r="J143" t="inlineStr"/>
       <c r="K143" t="inlineStr"/>
       <c r="L143" t="inlineStr"/>
@@ -4305,7 +4305,7 @@
       <c r="G144" t="inlineStr"/>
       <c r="H144" t="inlineStr"/>
       <c r="I144" t="n">
-        <v>703.41796875</v>
+        <v>4407.12890625</v>
       </c>
       <c r="J144" t="inlineStr"/>
       <c r="K144" t="inlineStr"/>
@@ -4321,7 +4321,7 @@
       <c r="G145" t="inlineStr"/>
       <c r="H145" t="inlineStr"/>
       <c r="I145" t="n">
-        <v>990.52734375</v>
+        <v>5555.56640625</v>
       </c>
       <c r="J145" t="inlineStr"/>
       <c r="K145" t="inlineStr"/>
@@ -4337,7 +4337,7 @@
       <c r="G146" t="inlineStr"/>
       <c r="H146" t="inlineStr"/>
       <c r="I146" t="n">
-        <v>1320.703125</v>
+        <v>6474.31640625</v>
       </c>
       <c r="J146" t="inlineStr"/>
       <c r="K146" t="inlineStr"/>
@@ -4353,7 +4353,7 @@
       <c r="G147" t="inlineStr"/>
       <c r="H147" t="inlineStr"/>
       <c r="I147" t="n">
-        <v>1679.58984375</v>
+        <v>7665.8203125</v>
       </c>
       <c r="J147" t="inlineStr"/>
       <c r="K147" t="inlineStr"/>
@@ -4369,7 +4369,7 @@
       <c r="G148" t="inlineStr"/>
       <c r="H148" t="inlineStr"/>
       <c r="I148" t="n">
-        <v>1780.078125</v>
+        <v>9115.72265625</v>
       </c>
       <c r="J148" t="inlineStr"/>
       <c r="K148" t="inlineStr"/>
@@ -4385,7 +4385,7 @@
       <c r="G149" t="inlineStr"/>
       <c r="H149" t="inlineStr"/>
       <c r="I149" t="n">
-        <v>1894.921875</v>
+        <v>11714.0625</v>
       </c>
       <c r="J149" t="inlineStr"/>
       <c r="K149" t="inlineStr"/>
@@ -4400,10 +4400,10 @@
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr"/>
       <c r="H150" t="inlineStr"/>
-      <c r="I150" t="n">
-        <v>2138.96484375</v>
-      </c>
-      <c r="J150" t="inlineStr"/>
+      <c r="I150" t="inlineStr"/>
+      <c r="J150" t="n">
+        <v>660.3515625</v>
+      </c>
       <c r="K150" t="inlineStr"/>
       <c r="L150" t="inlineStr"/>
     </row>
@@ -4416,10 +4416,10 @@
       <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr"/>
       <c r="H151" t="inlineStr"/>
-      <c r="I151" t="n">
-        <v>3258.69140625</v>
-      </c>
-      <c r="J151" t="inlineStr"/>
+      <c r="I151" t="inlineStr"/>
+      <c r="J151" t="n">
+        <v>904.39453125</v>
+      </c>
       <c r="K151" t="inlineStr"/>
       <c r="L151" t="inlineStr"/>
     </row>
@@ -4432,10 +4432,10 @@
       <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr"/>
       <c r="H152" t="inlineStr"/>
-      <c r="I152" t="n">
-        <v>3732.421875</v>
-      </c>
-      <c r="J152" t="inlineStr"/>
+      <c r="I152" t="inlineStr"/>
+      <c r="J152" t="n">
+        <v>976.171875</v>
+      </c>
       <c r="K152" t="inlineStr"/>
       <c r="L152" t="inlineStr"/>
     </row>
@@ -4448,10 +4448,10 @@
       <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr"/>
       <c r="H153" t="inlineStr"/>
-      <c r="I153" t="n">
-        <v>4163.0859375</v>
-      </c>
-      <c r="J153" t="inlineStr"/>
+      <c r="I153" t="inlineStr"/>
+      <c r="J153" t="n">
+        <v>1277.63671875</v>
+      </c>
       <c r="K153" t="inlineStr"/>
       <c r="L153" t="inlineStr"/>
     </row>
@@ -4464,10 +4464,10 @@
       <c r="F154" t="inlineStr"/>
       <c r="G154" t="inlineStr"/>
       <c r="H154" t="inlineStr"/>
-      <c r="I154" t="n">
-        <v>4407.12890625</v>
-      </c>
-      <c r="J154" t="inlineStr"/>
+      <c r="I154" t="inlineStr"/>
+      <c r="J154" t="n">
+        <v>1335.05859375</v>
+      </c>
       <c r="K154" t="inlineStr"/>
       <c r="L154" t="inlineStr"/>
     </row>
@@ -4480,10 +4480,10 @@
       <c r="F155" t="inlineStr"/>
       <c r="G155" t="inlineStr"/>
       <c r="H155" t="inlineStr"/>
-      <c r="I155" t="n">
-        <v>5555.56640625</v>
-      </c>
-      <c r="J155" t="inlineStr"/>
+      <c r="I155" t="inlineStr"/>
+      <c r="J155" t="n">
+        <v>1435.546875</v>
+      </c>
       <c r="K155" t="inlineStr"/>
       <c r="L155" t="inlineStr"/>
     </row>
@@ -4496,10 +4496,10 @@
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr"/>
       <c r="H156" t="inlineStr"/>
-      <c r="I156" t="n">
-        <v>6474.31640625</v>
-      </c>
-      <c r="J156" t="inlineStr"/>
+      <c r="I156" t="inlineStr"/>
+      <c r="J156" t="n">
+        <v>1521.6796875</v>
+      </c>
       <c r="K156" t="inlineStr"/>
       <c r="L156" t="inlineStr"/>
     </row>
@@ -4512,10 +4512,10 @@
       <c r="F157" t="inlineStr"/>
       <c r="G157" t="inlineStr"/>
       <c r="H157" t="inlineStr"/>
-      <c r="I157" t="n">
-        <v>7665.8203125</v>
-      </c>
-      <c r="J157" t="inlineStr"/>
+      <c r="I157" t="inlineStr"/>
+      <c r="J157" t="n">
+        <v>1665.234375</v>
+      </c>
       <c r="K157" t="inlineStr"/>
       <c r="L157" t="inlineStr"/>
     </row>
@@ -4528,10 +4528,10 @@
       <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr"/>
       <c r="H158" t="inlineStr"/>
-      <c r="I158" t="n">
-        <v>7895.5078125</v>
-      </c>
-      <c r="J158" t="inlineStr"/>
+      <c r="I158" t="inlineStr"/>
+      <c r="J158" t="n">
+        <v>1808.7890625</v>
+      </c>
       <c r="K158" t="inlineStr"/>
       <c r="L158" t="inlineStr"/>
     </row>
@@ -4544,10 +4544,10 @@
       <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr"/>
       <c r="H159" t="inlineStr"/>
-      <c r="I159" t="n">
-        <v>9115.72265625</v>
-      </c>
-      <c r="J159" t="inlineStr"/>
+      <c r="I159" t="inlineStr"/>
+      <c r="J159" t="n">
+        <v>1923.6328125</v>
+      </c>
       <c r="K159" t="inlineStr"/>
       <c r="L159" t="inlineStr"/>
     </row>
@@ -4560,10 +4560,10 @@
       <c r="F160" t="inlineStr"/>
       <c r="G160" t="inlineStr"/>
       <c r="H160" t="inlineStr"/>
-      <c r="I160" t="n">
-        <v>11714.0625</v>
-      </c>
-      <c r="J160" t="inlineStr"/>
+      <c r="I160" t="inlineStr"/>
+      <c r="J160" t="n">
+        <v>2038.4765625</v>
+      </c>
       <c r="K160" t="inlineStr"/>
       <c r="L160" t="inlineStr"/>
     </row>
@@ -4578,7 +4578,7 @@
       <c r="H161" t="inlineStr"/>
       <c r="I161" t="inlineStr"/>
       <c r="J161" t="n">
-        <v>660.3515625</v>
+        <v>2153.3203125</v>
       </c>
       <c r="K161" t="inlineStr"/>
       <c r="L161" t="inlineStr"/>
@@ -4594,7 +4594,7 @@
       <c r="H162" t="inlineStr"/>
       <c r="I162" t="inlineStr"/>
       <c r="J162" t="n">
-        <v>861.328125</v>
+        <v>2282.51953125</v>
       </c>
       <c r="K162" t="inlineStr"/>
       <c r="L162" t="inlineStr"/>
@@ -4610,7 +4610,7 @@
       <c r="H163" t="inlineStr"/>
       <c r="I163" t="inlineStr"/>
       <c r="J163" t="n">
-        <v>904.39453125</v>
+        <v>2698.828125</v>
       </c>
       <c r="K163" t="inlineStr"/>
       <c r="L163" t="inlineStr"/>
@@ -4626,7 +4626,7 @@
       <c r="H164" t="inlineStr"/>
       <c r="I164" t="inlineStr"/>
       <c r="J164" t="n">
-        <v>976.171875</v>
+        <v>2842.3828125</v>
       </c>
       <c r="K164" t="inlineStr"/>
       <c r="L164" t="inlineStr"/>
@@ -4642,7 +4642,7 @@
       <c r="H165" t="inlineStr"/>
       <c r="I165" t="inlineStr"/>
       <c r="J165" t="n">
-        <v>1033.59375</v>
+        <v>3631.93359375</v>
       </c>
       <c r="K165" t="inlineStr"/>
       <c r="L165" t="inlineStr"/>
@@ -4658,7 +4658,7 @@
       <c r="H166" t="inlineStr"/>
       <c r="I166" t="inlineStr"/>
       <c r="J166" t="n">
-        <v>1091.015625</v>
+        <v>6043.65234375</v>
       </c>
       <c r="K166" t="inlineStr"/>
       <c r="L166" t="inlineStr"/>
@@ -4674,7 +4674,7 @@
       <c r="H167" t="inlineStr"/>
       <c r="I167" t="inlineStr"/>
       <c r="J167" t="n">
-        <v>1277.63671875</v>
+        <v>7278.22265625</v>
       </c>
       <c r="K167" t="inlineStr"/>
       <c r="L167" t="inlineStr"/>
@@ -4689,10 +4689,10 @@
       <c r="G168" t="inlineStr"/>
       <c r="H168" t="inlineStr"/>
       <c r="I168" t="inlineStr"/>
-      <c r="J168" t="n">
-        <v>1335.05859375</v>
-      </c>
-      <c r="K168" t="inlineStr"/>
+      <c r="J168" t="inlineStr"/>
+      <c r="K168" t="n">
+        <v>602.9296875</v>
+      </c>
       <c r="L168" t="inlineStr"/>
     </row>
     <row r="169">
@@ -4705,10 +4705,10 @@
       <c r="G169" t="inlineStr"/>
       <c r="H169" t="inlineStr"/>
       <c r="I169" t="inlineStr"/>
-      <c r="J169" t="n">
-        <v>1435.546875</v>
-      </c>
-      <c r="K169" t="inlineStr"/>
+      <c r="J169" t="inlineStr"/>
+      <c r="K169" t="n">
+        <v>861.328125</v>
+      </c>
       <c r="L169" t="inlineStr"/>
     </row>
     <row r="170">
@@ -4721,10 +4721,10 @@
       <c r="G170" t="inlineStr"/>
       <c r="H170" t="inlineStr"/>
       <c r="I170" t="inlineStr"/>
-      <c r="J170" t="n">
-        <v>1521.6796875</v>
-      </c>
-      <c r="K170" t="inlineStr"/>
+      <c r="J170" t="inlineStr"/>
+      <c r="K170" t="n">
+        <v>933.10546875</v>
+      </c>
       <c r="L170" t="inlineStr"/>
     </row>
     <row r="171">
@@ -4737,10 +4737,10 @@
       <c r="G171" t="inlineStr"/>
       <c r="H171" t="inlineStr"/>
       <c r="I171" t="inlineStr"/>
-      <c r="J171" t="n">
-        <v>1665.234375</v>
-      </c>
-      <c r="K171" t="inlineStr"/>
+      <c r="J171" t="inlineStr"/>
+      <c r="K171" t="n">
+        <v>1263.28125</v>
+      </c>
       <c r="L171" t="inlineStr"/>
     </row>
     <row r="172">
@@ -4753,10 +4753,10 @@
       <c r="G172" t="inlineStr"/>
       <c r="H172" t="inlineStr"/>
       <c r="I172" t="inlineStr"/>
-      <c r="J172" t="n">
-        <v>1808.7890625</v>
-      </c>
-      <c r="K172" t="inlineStr"/>
+      <c r="J172" t="inlineStr"/>
+      <c r="K172" t="n">
+        <v>1349.4140625</v>
+      </c>
       <c r="L172" t="inlineStr"/>
     </row>
     <row r="173">
@@ -4769,10 +4769,10 @@
       <c r="G173" t="inlineStr"/>
       <c r="H173" t="inlineStr"/>
       <c r="I173" t="inlineStr"/>
-      <c r="J173" t="n">
-        <v>1923.6328125</v>
-      </c>
-      <c r="K173" t="inlineStr"/>
+      <c r="J173" t="inlineStr"/>
+      <c r="K173" t="n">
+        <v>1536.03515625</v>
+      </c>
       <c r="L173" t="inlineStr"/>
     </row>
     <row r="174">
@@ -4785,10 +4785,10 @@
       <c r="G174" t="inlineStr"/>
       <c r="H174" t="inlineStr"/>
       <c r="I174" t="inlineStr"/>
-      <c r="J174" t="n">
-        <v>2038.4765625</v>
-      </c>
-      <c r="K174" t="inlineStr"/>
+      <c r="J174" t="inlineStr"/>
+      <c r="K174" t="n">
+        <v>1622.16796875</v>
+      </c>
       <c r="L174" t="inlineStr"/>
     </row>
     <row r="175">
@@ -4801,10 +4801,10 @@
       <c r="G175" t="inlineStr"/>
       <c r="H175" t="inlineStr"/>
       <c r="I175" t="inlineStr"/>
-      <c r="J175" t="n">
-        <v>2153.3203125</v>
-      </c>
-      <c r="K175" t="inlineStr"/>
+      <c r="J175" t="inlineStr"/>
+      <c r="K175" t="n">
+        <v>2253.80859375</v>
+      </c>
       <c r="L175" t="inlineStr"/>
     </row>
     <row r="176">
@@ -4817,10 +4817,10 @@
       <c r="G176" t="inlineStr"/>
       <c r="H176" t="inlineStr"/>
       <c r="I176" t="inlineStr"/>
-      <c r="J176" t="n">
-        <v>2282.51953125</v>
-      </c>
-      <c r="K176" t="inlineStr"/>
+      <c r="J176" t="inlineStr"/>
+      <c r="K176" t="n">
+        <v>2828.02734375</v>
+      </c>
       <c r="L176" t="inlineStr"/>
     </row>
     <row r="177">
@@ -4833,10 +4833,10 @@
       <c r="G177" t="inlineStr"/>
       <c r="H177" t="inlineStr"/>
       <c r="I177" t="inlineStr"/>
-      <c r="J177" t="n">
-        <v>2698.828125</v>
-      </c>
-      <c r="K177" t="inlineStr"/>
+      <c r="J177" t="inlineStr"/>
+      <c r="K177" t="n">
+        <v>3086.42578125</v>
+      </c>
       <c r="L177" t="inlineStr"/>
     </row>
     <row r="178">
@@ -4849,10 +4849,10 @@
       <c r="G178" t="inlineStr"/>
       <c r="H178" t="inlineStr"/>
       <c r="I178" t="inlineStr"/>
-      <c r="J178" t="n">
-        <v>2842.3828125</v>
-      </c>
-      <c r="K178" t="inlineStr"/>
+      <c r="J178" t="inlineStr"/>
+      <c r="K178" t="n">
+        <v>3445.3125</v>
+      </c>
       <c r="L178" t="inlineStr"/>
     </row>
     <row r="179">
@@ -4865,10 +4865,10 @@
       <c r="G179" t="inlineStr"/>
       <c r="H179" t="inlineStr"/>
       <c r="I179" t="inlineStr"/>
-      <c r="J179" t="n">
-        <v>3631.93359375</v>
-      </c>
-      <c r="K179" t="inlineStr"/>
+      <c r="J179" t="inlineStr"/>
+      <c r="K179" t="n">
+        <v>4378.41796875</v>
+      </c>
       <c r="L179" t="inlineStr"/>
     </row>
     <row r="180">
@@ -4881,10 +4881,10 @@
       <c r="G180" t="inlineStr"/>
       <c r="H180" t="inlineStr"/>
       <c r="I180" t="inlineStr"/>
-      <c r="J180" t="n">
-        <v>6043.65234375</v>
-      </c>
-      <c r="K180" t="inlineStr"/>
+      <c r="J180" t="inlineStr"/>
+      <c r="K180" t="n">
+        <v>4521.97265625</v>
+      </c>
       <c r="L180" t="inlineStr"/>
     </row>
     <row r="181">
@@ -4897,10 +4897,10 @@
       <c r="G181" t="inlineStr"/>
       <c r="H181" t="inlineStr"/>
       <c r="I181" t="inlineStr"/>
-      <c r="J181" t="n">
-        <v>7278.22265625</v>
-      </c>
-      <c r="K181" t="inlineStr"/>
+      <c r="J181" t="inlineStr"/>
+      <c r="K181" t="n">
+        <v>4722.94921875</v>
+      </c>
       <c r="L181" t="inlineStr"/>
     </row>
     <row r="182">
@@ -4915,7 +4915,7 @@
       <c r="I182" t="inlineStr"/>
       <c r="J182" t="inlineStr"/>
       <c r="K182" t="n">
-        <v>602.9296875</v>
+        <v>6058.0078125</v>
       </c>
       <c r="L182" t="inlineStr"/>
     </row>
@@ -4931,7 +4931,7 @@
       <c r="I183" t="inlineStr"/>
       <c r="J183" t="inlineStr"/>
       <c r="K183" t="n">
-        <v>660.3515625</v>
+        <v>6316.40625</v>
       </c>
       <c r="L183" t="inlineStr"/>
     </row>
@@ -4946,10 +4946,10 @@
       <c r="H184" t="inlineStr"/>
       <c r="I184" t="inlineStr"/>
       <c r="J184" t="inlineStr"/>
-      <c r="K184" t="n">
-        <v>861.328125</v>
-      </c>
-      <c r="L184" t="inlineStr"/>
+      <c r="K184" t="inlineStr"/>
+      <c r="L184" t="n">
+        <v>1406.8359375</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr"/>
@@ -4962,10 +4962,10 @@
       <c r="H185" t="inlineStr"/>
       <c r="I185" t="inlineStr"/>
       <c r="J185" t="inlineStr"/>
-      <c r="K185" t="n">
-        <v>933.10546875</v>
-      </c>
-      <c r="L185" t="inlineStr"/>
+      <c r="K185" t="inlineStr"/>
+      <c r="L185" t="n">
+        <v>1507.32421875</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr"/>
@@ -4978,10 +4978,10 @@
       <c r="H186" t="inlineStr"/>
       <c r="I186" t="inlineStr"/>
       <c r="J186" t="inlineStr"/>
-      <c r="K186" t="n">
-        <v>1119.7265625</v>
-      </c>
-      <c r="L186" t="inlineStr"/>
+      <c r="K186" t="inlineStr"/>
+      <c r="L186" t="n">
+        <v>1622.16796875</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr"/>
@@ -4994,10 +4994,10 @@
       <c r="H187" t="inlineStr"/>
       <c r="I187" t="inlineStr"/>
       <c r="J187" t="inlineStr"/>
-      <c r="K187" t="n">
-        <v>1191.50390625</v>
-      </c>
-      <c r="L187" t="inlineStr"/>
+      <c r="K187" t="inlineStr"/>
+      <c r="L187" t="n">
+        <v>1722.65625</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr"/>
@@ -5010,10 +5010,10 @@
       <c r="H188" t="inlineStr"/>
       <c r="I188" t="inlineStr"/>
       <c r="J188" t="inlineStr"/>
-      <c r="K188" t="n">
-        <v>1263.28125</v>
-      </c>
-      <c r="L188" t="inlineStr"/>
+      <c r="K188" t="inlineStr"/>
+      <c r="L188" t="n">
+        <v>1880.56640625</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr"/>
@@ -5026,10 +5026,10 @@
       <c r="H189" t="inlineStr"/>
       <c r="I189" t="inlineStr"/>
       <c r="J189" t="inlineStr"/>
-      <c r="K189" t="n">
-        <v>1349.4140625</v>
-      </c>
-      <c r="L189" t="inlineStr"/>
+      <c r="K189" t="inlineStr"/>
+      <c r="L189" t="n">
+        <v>2009.765625</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr"/>
@@ -5042,10 +5042,10 @@
       <c r="H190" t="inlineStr"/>
       <c r="I190" t="inlineStr"/>
       <c r="J190" t="inlineStr"/>
-      <c r="K190" t="n">
-        <v>1435.546875</v>
-      </c>
-      <c r="L190" t="inlineStr"/>
+      <c r="K190" t="inlineStr"/>
+      <c r="L190" t="n">
+        <v>2138.96484375</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr"/>
@@ -5058,10 +5058,10 @@
       <c r="H191" t="inlineStr"/>
       <c r="I191" t="inlineStr"/>
       <c r="J191" t="inlineStr"/>
-      <c r="K191" t="n">
-        <v>1536.03515625</v>
-      </c>
-      <c r="L191" t="inlineStr"/>
+      <c r="K191" t="inlineStr"/>
+      <c r="L191" t="n">
+        <v>2296.875</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr"/>
@@ -5074,10 +5074,10 @@
       <c r="H192" t="inlineStr"/>
       <c r="I192" t="inlineStr"/>
       <c r="J192" t="inlineStr"/>
-      <c r="K192" t="n">
-        <v>1622.16796875</v>
-      </c>
-      <c r="L192" t="inlineStr"/>
+      <c r="K192" t="inlineStr"/>
+      <c r="L192" t="n">
+        <v>2469.140625</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr"/>
@@ -5090,10 +5090,10 @@
       <c r="H193" t="inlineStr"/>
       <c r="I193" t="inlineStr"/>
       <c r="J193" t="inlineStr"/>
-      <c r="K193" t="n">
-        <v>2253.80859375</v>
-      </c>
-      <c r="L193" t="inlineStr"/>
+      <c r="K193" t="inlineStr"/>
+      <c r="L193" t="n">
+        <v>2612.6953125</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr"/>
@@ -5106,10 +5106,10 @@
       <c r="H194" t="inlineStr"/>
       <c r="I194" t="inlineStr"/>
       <c r="J194" t="inlineStr"/>
-      <c r="K194" t="n">
-        <v>2828.02734375</v>
-      </c>
-      <c r="L194" t="inlineStr"/>
+      <c r="K194" t="inlineStr"/>
+      <c r="L194" t="n">
+        <v>2756.25</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr"/>
@@ -5122,10 +5122,10 @@
       <c r="H195" t="inlineStr"/>
       <c r="I195" t="inlineStr"/>
       <c r="J195" t="inlineStr"/>
-      <c r="K195" t="n">
-        <v>3086.42578125</v>
-      </c>
-      <c r="L195" t="inlineStr"/>
+      <c r="K195" t="inlineStr"/>
+      <c r="L195" t="n">
+        <v>2914.16015625</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr"/>
@@ -5138,10 +5138,10 @@
       <c r="H196" t="inlineStr"/>
       <c r="I196" t="inlineStr"/>
       <c r="J196" t="inlineStr"/>
-      <c r="K196" t="n">
-        <v>3445.3125</v>
-      </c>
-      <c r="L196" t="inlineStr"/>
+      <c r="K196" t="inlineStr"/>
+      <c r="L196" t="n">
+        <v>3072.0703125</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr"/>
@@ -5154,10 +5154,10 @@
       <c r="H197" t="inlineStr"/>
       <c r="I197" t="inlineStr"/>
       <c r="J197" t="inlineStr"/>
-      <c r="K197" t="n">
-        <v>4378.41796875</v>
-      </c>
-      <c r="L197" t="inlineStr"/>
+      <c r="K197" t="inlineStr"/>
+      <c r="L197" t="n">
+        <v>3273.046875</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr"/>
@@ -5170,296 +5170,8 @@
       <c r="H198" t="inlineStr"/>
       <c r="I198" t="inlineStr"/>
       <c r="J198" t="inlineStr"/>
-      <c r="K198" t="n">
-        <v>4521.97265625</v>
-      </c>
-      <c r="L198" t="inlineStr"/>
-    </row>
-    <row r="199">
-      <c r="A199" t="inlineStr"/>
-      <c r="B199" t="inlineStr"/>
-      <c r="C199" t="inlineStr"/>
-      <c r="D199" t="inlineStr"/>
-      <c r="E199" t="inlineStr"/>
-      <c r="F199" t="inlineStr"/>
-      <c r="G199" t="inlineStr"/>
-      <c r="H199" t="inlineStr"/>
-      <c r="I199" t="inlineStr"/>
-      <c r="J199" t="inlineStr"/>
-      <c r="K199" t="n">
-        <v>4722.94921875</v>
-      </c>
-      <c r="L199" t="inlineStr"/>
-    </row>
-    <row r="200">
-      <c r="A200" t="inlineStr"/>
-      <c r="B200" t="inlineStr"/>
-      <c r="C200" t="inlineStr"/>
-      <c r="D200" t="inlineStr"/>
-      <c r="E200" t="inlineStr"/>
-      <c r="F200" t="inlineStr"/>
-      <c r="G200" t="inlineStr"/>
-      <c r="H200" t="inlineStr"/>
-      <c r="I200" t="inlineStr"/>
-      <c r="J200" t="inlineStr"/>
-      <c r="K200" t="n">
-        <v>6058.0078125</v>
-      </c>
-      <c r="L200" t="inlineStr"/>
-    </row>
-    <row r="201">
-      <c r="A201" t="inlineStr"/>
-      <c r="B201" t="inlineStr"/>
-      <c r="C201" t="inlineStr"/>
-      <c r="D201" t="inlineStr"/>
-      <c r="E201" t="inlineStr"/>
-      <c r="F201" t="inlineStr"/>
-      <c r="G201" t="inlineStr"/>
-      <c r="H201" t="inlineStr"/>
-      <c r="I201" t="inlineStr"/>
-      <c r="J201" t="inlineStr"/>
-      <c r="K201" t="n">
-        <v>6316.40625</v>
-      </c>
-      <c r="L201" t="inlineStr"/>
-    </row>
-    <row r="202">
-      <c r="A202" t="inlineStr"/>
-      <c r="B202" t="inlineStr"/>
-      <c r="C202" t="inlineStr"/>
-      <c r="D202" t="inlineStr"/>
-      <c r="E202" t="inlineStr"/>
-      <c r="F202" t="inlineStr"/>
-      <c r="G202" t="inlineStr"/>
-      <c r="H202" t="inlineStr"/>
-      <c r="I202" t="inlineStr"/>
-      <c r="J202" t="inlineStr"/>
-      <c r="K202" t="inlineStr"/>
-      <c r="L202" t="n">
-        <v>1406.8359375</v>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" t="inlineStr"/>
-      <c r="B203" t="inlineStr"/>
-      <c r="C203" t="inlineStr"/>
-      <c r="D203" t="inlineStr"/>
-      <c r="E203" t="inlineStr"/>
-      <c r="F203" t="inlineStr"/>
-      <c r="G203" t="inlineStr"/>
-      <c r="H203" t="inlineStr"/>
-      <c r="I203" t="inlineStr"/>
-      <c r="J203" t="inlineStr"/>
-      <c r="K203" t="inlineStr"/>
-      <c r="L203" t="n">
-        <v>1507.32421875</v>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" t="inlineStr"/>
-      <c r="B204" t="inlineStr"/>
-      <c r="C204" t="inlineStr"/>
-      <c r="D204" t="inlineStr"/>
-      <c r="E204" t="inlineStr"/>
-      <c r="F204" t="inlineStr"/>
-      <c r="G204" t="inlineStr"/>
-      <c r="H204" t="inlineStr"/>
-      <c r="I204" t="inlineStr"/>
-      <c r="J204" t="inlineStr"/>
-      <c r="K204" t="inlineStr"/>
-      <c r="L204" t="n">
-        <v>1622.16796875</v>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" t="inlineStr"/>
-      <c r="B205" t="inlineStr"/>
-      <c r="C205" t="inlineStr"/>
-      <c r="D205" t="inlineStr"/>
-      <c r="E205" t="inlineStr"/>
-      <c r="F205" t="inlineStr"/>
-      <c r="G205" t="inlineStr"/>
-      <c r="H205" t="inlineStr"/>
-      <c r="I205" t="inlineStr"/>
-      <c r="J205" t="inlineStr"/>
-      <c r="K205" t="inlineStr"/>
-      <c r="L205" t="n">
-        <v>1722.65625</v>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" t="inlineStr"/>
-      <c r="B206" t="inlineStr"/>
-      <c r="C206" t="inlineStr"/>
-      <c r="D206" t="inlineStr"/>
-      <c r="E206" t="inlineStr"/>
-      <c r="F206" t="inlineStr"/>
-      <c r="G206" t="inlineStr"/>
-      <c r="H206" t="inlineStr"/>
-      <c r="I206" t="inlineStr"/>
-      <c r="J206" t="inlineStr"/>
-      <c r="K206" t="inlineStr"/>
-      <c r="L206" t="n">
-        <v>1880.56640625</v>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" t="inlineStr"/>
-      <c r="B207" t="inlineStr"/>
-      <c r="C207" t="inlineStr"/>
-      <c r="D207" t="inlineStr"/>
-      <c r="E207" t="inlineStr"/>
-      <c r="F207" t="inlineStr"/>
-      <c r="G207" t="inlineStr"/>
-      <c r="H207" t="inlineStr"/>
-      <c r="I207" t="inlineStr"/>
-      <c r="J207" t="inlineStr"/>
-      <c r="K207" t="inlineStr"/>
-      <c r="L207" t="n">
-        <v>2009.765625</v>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" t="inlineStr"/>
-      <c r="B208" t="inlineStr"/>
-      <c r="C208" t="inlineStr"/>
-      <c r="D208" t="inlineStr"/>
-      <c r="E208" t="inlineStr"/>
-      <c r="F208" t="inlineStr"/>
-      <c r="G208" t="inlineStr"/>
-      <c r="H208" t="inlineStr"/>
-      <c r="I208" t="inlineStr"/>
-      <c r="J208" t="inlineStr"/>
-      <c r="K208" t="inlineStr"/>
-      <c r="L208" t="n">
-        <v>2138.96484375</v>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" t="inlineStr"/>
-      <c r="B209" t="inlineStr"/>
-      <c r="C209" t="inlineStr"/>
-      <c r="D209" t="inlineStr"/>
-      <c r="E209" t="inlineStr"/>
-      <c r="F209" t="inlineStr"/>
-      <c r="G209" t="inlineStr"/>
-      <c r="H209" t="inlineStr"/>
-      <c r="I209" t="inlineStr"/>
-      <c r="J209" t="inlineStr"/>
-      <c r="K209" t="inlineStr"/>
-      <c r="L209" t="n">
-        <v>2296.875</v>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" t="inlineStr"/>
-      <c r="B210" t="inlineStr"/>
-      <c r="C210" t="inlineStr"/>
-      <c r="D210" t="inlineStr"/>
-      <c r="E210" t="inlineStr"/>
-      <c r="F210" t="inlineStr"/>
-      <c r="G210" t="inlineStr"/>
-      <c r="H210" t="inlineStr"/>
-      <c r="I210" t="inlineStr"/>
-      <c r="J210" t="inlineStr"/>
-      <c r="K210" t="inlineStr"/>
-      <c r="L210" t="n">
-        <v>2469.140625</v>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" t="inlineStr"/>
-      <c r="B211" t="inlineStr"/>
-      <c r="C211" t="inlineStr"/>
-      <c r="D211" t="inlineStr"/>
-      <c r="E211" t="inlineStr"/>
-      <c r="F211" t="inlineStr"/>
-      <c r="G211" t="inlineStr"/>
-      <c r="H211" t="inlineStr"/>
-      <c r="I211" t="inlineStr"/>
-      <c r="J211" t="inlineStr"/>
-      <c r="K211" t="inlineStr"/>
-      <c r="L211" t="n">
-        <v>2612.6953125</v>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" t="inlineStr"/>
-      <c r="B212" t="inlineStr"/>
-      <c r="C212" t="inlineStr"/>
-      <c r="D212" t="inlineStr"/>
-      <c r="E212" t="inlineStr"/>
-      <c r="F212" t="inlineStr"/>
-      <c r="G212" t="inlineStr"/>
-      <c r="H212" t="inlineStr"/>
-      <c r="I212" t="inlineStr"/>
-      <c r="J212" t="inlineStr"/>
-      <c r="K212" t="inlineStr"/>
-      <c r="L212" t="n">
-        <v>2756.25</v>
-      </c>
-    </row>
-    <row r="213">
-      <c r="A213" t="inlineStr"/>
-      <c r="B213" t="inlineStr"/>
-      <c r="C213" t="inlineStr"/>
-      <c r="D213" t="inlineStr"/>
-      <c r="E213" t="inlineStr"/>
-      <c r="F213" t="inlineStr"/>
-      <c r="G213" t="inlineStr"/>
-      <c r="H213" t="inlineStr"/>
-      <c r="I213" t="inlineStr"/>
-      <c r="J213" t="inlineStr"/>
-      <c r="K213" t="inlineStr"/>
-      <c r="L213" t="n">
-        <v>2914.16015625</v>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" t="inlineStr"/>
-      <c r="B214" t="inlineStr"/>
-      <c r="C214" t="inlineStr"/>
-      <c r="D214" t="inlineStr"/>
-      <c r="E214" t="inlineStr"/>
-      <c r="F214" t="inlineStr"/>
-      <c r="G214" t="inlineStr"/>
-      <c r="H214" t="inlineStr"/>
-      <c r="I214" t="inlineStr"/>
-      <c r="J214" t="inlineStr"/>
-      <c r="K214" t="inlineStr"/>
-      <c r="L214" t="n">
-        <v>3072.0703125</v>
-      </c>
-    </row>
-    <row r="215">
-      <c r="A215" t="inlineStr"/>
-      <c r="B215" t="inlineStr"/>
-      <c r="C215" t="inlineStr"/>
-      <c r="D215" t="inlineStr"/>
-      <c r="E215" t="inlineStr"/>
-      <c r="F215" t="inlineStr"/>
-      <c r="G215" t="inlineStr"/>
-      <c r="H215" t="inlineStr"/>
-      <c r="I215" t="inlineStr"/>
-      <c r="J215" t="inlineStr"/>
-      <c r="K215" t="inlineStr"/>
-      <c r="L215" t="n">
-        <v>3273.046875</v>
-      </c>
-    </row>
-    <row r="216">
-      <c r="A216" t="inlineStr"/>
-      <c r="B216" t="inlineStr"/>
-      <c r="C216" t="inlineStr"/>
-      <c r="D216" t="inlineStr"/>
-      <c r="E216" t="inlineStr"/>
-      <c r="F216" t="inlineStr"/>
-      <c r="G216" t="inlineStr"/>
-      <c r="H216" t="inlineStr"/>
-      <c r="I216" t="inlineStr"/>
-      <c r="J216" t="inlineStr"/>
-      <c r="K216" t="inlineStr"/>
-      <c r="L216" t="n">
+      <c r="K198" t="inlineStr"/>
+      <c r="L198" t="n">
         <v>4134.375</v>
       </c>
     </row>

</xml_diff>

<commit_message>
final(?) analysese, still editing figures
</commit_message>
<xml_diff>
--- a/results/pp_human/Additional Human Picked Peaks [v3, scipy, prom_C=3, prom_mag=2, hpf_meth=HPF=(300Hz cf, 50Hz df, 100dB rip), fs=44100, tau=69.66ms, xi=15.08ms, hop_C=hop_mag=10.0ms, rho=1.0, hann, win_mag=hann, avg_meth=power, flim=[500, inf], wf_len_s=None].xlsx
+++ b/results/pp_human/Additional Human Picked Peaks [v3, scipy, prom_C=3, prom_mag=2, hpf_meth=HPF=(300Hz cf, 50Hz df, 100dB rip), fs=44100, tau=69.66ms, xi=15.08ms, hop_C=hop_mag=10.0ms, rho=1.0, hann, win_mag=hann, avg_meth=power, flim=[500, inf], wf_len_s=None].xlsx
@@ -1958,7 +1958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L198"/>
+  <dimension ref="A1:L202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2025,7 +2025,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>588.57421875</v>
+        <v>531.15234375</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
@@ -2041,7 +2041,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>631.640625</v>
+        <v>588.57421875</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
@@ -2057,7 +2057,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>689.0625</v>
+        <v>631.640625</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
@@ -2073,7 +2073,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>789.55078125</v>
+        <v>689.0625</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
@@ -2089,7 +2089,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>861.328125</v>
+        <v>789.55078125</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
@@ -2105,7 +2105,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>1177.1484375</v>
+        <v>861.328125</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
@@ -2121,7 +2121,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>1263.28125</v>
+        <v>1177.1484375</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
@@ -2137,7 +2137,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1363.76953125</v>
+        <v>1263.28125</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
@@ -2153,7 +2153,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1665.234375</v>
+        <v>1363.76953125</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
@@ -2169,7 +2169,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>1780.078125</v>
+        <v>1665.234375</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
@@ -2185,7 +2185,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>2038.4765625</v>
+        <v>1780.078125</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
@@ -2201,7 +2201,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>2167.67578125</v>
+        <v>2038.4765625</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
@@ -2217,7 +2217,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>2282.51953125</v>
+        <v>2167.67578125</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
@@ -2233,7 +2233,7 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>2397.36328125</v>
+        <v>2282.51953125</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
@@ -2249,7 +2249,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>2540.91796875</v>
+        <v>2397.36328125</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
@@ -2265,7 +2265,7 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>2698.828125</v>
+        <v>2540.91796875</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>2928.515625</v>
+        <v>2698.828125</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
@@ -2297,7 +2297,7 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>3115.13671875</v>
+        <v>2928.515625</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
@@ -2313,7 +2313,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>3718.06640625</v>
+        <v>3115.13671875</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
@@ -2329,7 +2329,7 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>3919.04296875</v>
+        <v>3718.06640625</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
@@ -2344,10 +2344,10 @@
       <c r="L21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
-      <c r="B22" t="n">
-        <v>689.0625</v>
-      </c>
+      <c r="A22" t="n">
+        <v>3919.04296875</v>
+      </c>
+      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
@@ -2362,7 +2362,7 @@
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="n">
-        <v>846.97265625</v>
+        <v>689.0625</v>
       </c>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
@@ -2378,7 +2378,7 @@
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="n">
-        <v>1263.28125</v>
+        <v>846.97265625</v>
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
@@ -2394,7 +2394,7 @@
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="n">
-        <v>1363.76953125</v>
+        <v>1263.28125</v>
       </c>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
@@ -2410,7 +2410,7 @@
     <row r="26">
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="n">
-        <v>1564.74609375</v>
+        <v>1363.76953125</v>
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
@@ -2426,7 +2426,7 @@
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="n">
-        <v>1708.30078125</v>
+        <v>1564.74609375</v>
       </c>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
@@ -2442,7 +2442,7 @@
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="n">
-        <v>1851.85546875</v>
+        <v>1708.30078125</v>
       </c>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
@@ -2458,7 +2458,7 @@
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="n">
-        <v>1995.41015625</v>
+        <v>1851.85546875</v>
       </c>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
@@ -2474,7 +2474,7 @@
     <row r="30">
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="n">
-        <v>2110.25390625</v>
+        <v>1995.41015625</v>
       </c>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
@@ -2490,7 +2490,7 @@
     <row r="31">
       <c r="A31" t="inlineStr"/>
       <c r="B31" t="n">
-        <v>2239.453125</v>
+        <v>2110.25390625</v>
       </c>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
@@ -2506,7 +2506,7 @@
     <row r="32">
       <c r="A32" t="inlineStr"/>
       <c r="B32" t="n">
-        <v>2411.71875</v>
+        <v>2239.453125</v>
       </c>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
@@ -2522,7 +2522,7 @@
     <row r="33">
       <c r="A33" t="inlineStr"/>
       <c r="B33" t="n">
-        <v>2454.78515625</v>
+        <v>2411.71875</v>
       </c>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
@@ -2538,7 +2538,7 @@
     <row r="34">
       <c r="A34" t="inlineStr"/>
       <c r="B34" t="n">
-        <v>2641.40625</v>
+        <v>2454.78515625</v>
       </c>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
@@ -2554,7 +2554,7 @@
     <row r="35">
       <c r="A35" t="inlineStr"/>
       <c r="B35" t="n">
-        <v>2985.9375</v>
+        <v>2641.40625</v>
       </c>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr"/>
@@ -2570,7 +2570,7 @@
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="n">
-        <v>3545.80078125</v>
+        <v>2985.9375</v>
       </c>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
@@ -2586,7 +2586,7 @@
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="n">
-        <v>4349.70703125</v>
+        <v>3545.80078125</v>
       </c>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
@@ -2602,7 +2602,7 @@
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="n">
-        <v>6574.8046875</v>
+        <v>4349.70703125</v>
       </c>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
@@ -2617,10 +2617,10 @@
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
-      <c r="B39" t="inlineStr"/>
-      <c r="C39" t="n">
-        <v>617.28515625</v>
-      </c>
+      <c r="B39" t="n">
+        <v>6574.8046875</v>
+      </c>
+      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr"/>
@@ -2635,7 +2635,7 @@
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="n">
-        <v>732.12890625</v>
+        <v>617.28515625</v>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr"/>
@@ -2651,7 +2651,7 @@
       <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="n">
-        <v>803.90625</v>
+        <v>732.12890625</v>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr"/>
@@ -2667,7 +2667,7 @@
       <c r="A42" t="inlineStr"/>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="n">
-        <v>918.75</v>
+        <v>803.90625</v>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr"/>
@@ -2683,7 +2683,7 @@
       <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="n">
-        <v>990.52734375</v>
+        <v>918.75</v>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr"/>
@@ -2699,7 +2699,7 @@
       <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="n">
-        <v>1076.66015625</v>
+        <v>990.52734375</v>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr"/>
@@ -2715,7 +2715,7 @@
       <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="n">
-        <v>1134.08203125</v>
+        <v>1076.66015625</v>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr"/>
@@ -2731,7 +2731,7 @@
       <c r="A46" t="inlineStr"/>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="n">
-        <v>1263.28125</v>
+        <v>1134.08203125</v>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr"/>
@@ -2747,7 +2747,7 @@
       <c r="A47" t="inlineStr"/>
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="n">
-        <v>1320.703125</v>
+        <v>1263.28125</v>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr"/>
@@ -2763,7 +2763,7 @@
       <c r="A48" t="inlineStr"/>
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="n">
-        <v>1449.90234375</v>
+        <v>1320.703125</v>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr"/>
@@ -2779,7 +2779,7 @@
       <c r="A49" t="inlineStr"/>
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="n">
-        <v>1507.32421875</v>
+        <v>1449.90234375</v>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr"/>
@@ -2795,7 +2795,7 @@
       <c r="A50" t="inlineStr"/>
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="n">
-        <v>1579.1015625</v>
+        <v>1507.32421875</v>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr"/>
@@ -2811,7 +2811,7 @@
       <c r="A51" t="inlineStr"/>
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="n">
-        <v>1665.234375</v>
+        <v>1579.1015625</v>
       </c>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr"/>
@@ -2827,7 +2827,7 @@
       <c r="A52" t="inlineStr"/>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="n">
-        <v>1737.01171875</v>
+        <v>1665.234375</v>
       </c>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr"/>
@@ -2843,7 +2843,7 @@
       <c r="A53" t="inlineStr"/>
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="n">
-        <v>1794.43359375</v>
+        <v>1737.01171875</v>
       </c>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr"/>
@@ -2859,7 +2859,7 @@
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="n">
-        <v>2268.1640625</v>
+        <v>1794.43359375</v>
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr"/>
@@ -2875,7 +2875,7 @@
       <c r="A55" t="inlineStr"/>
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="n">
-        <v>3646.2890625</v>
+        <v>2268.1640625</v>
       </c>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr"/>
@@ -2891,7 +2891,7 @@
       <c r="A56" t="inlineStr"/>
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="n">
-        <v>3861.62109375</v>
+        <v>3646.2890625</v>
       </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr"/>
@@ -2907,7 +2907,7 @@
       <c r="A57" t="inlineStr"/>
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="n">
-        <v>4019.53125</v>
+        <v>3861.62109375</v>
       </c>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr"/>
@@ -2923,7 +2923,7 @@
       <c r="A58" t="inlineStr"/>
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="n">
-        <v>4177.44140625</v>
+        <v>4019.53125</v>
       </c>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr"/>
@@ -2939,7 +2939,7 @@
       <c r="A59" t="inlineStr"/>
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="n">
-        <v>4694.23828125</v>
+        <v>4177.44140625</v>
       </c>
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr"/>
@@ -2955,7 +2955,7 @@
       <c r="A60" t="inlineStr"/>
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="n">
-        <v>5656.0546875</v>
+        <v>4694.23828125</v>
       </c>
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr"/>
@@ -2971,7 +2971,7 @@
       <c r="A61" t="inlineStr"/>
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="n">
-        <v>6761.42578125</v>
+        <v>5656.0546875</v>
       </c>
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr"/>
@@ -2987,7 +2987,7 @@
       <c r="A62" t="inlineStr"/>
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="n">
-        <v>7048.53515625</v>
+        <v>6761.42578125</v>
       </c>
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr"/>
@@ -3003,7 +3003,7 @@
       <c r="A63" t="inlineStr"/>
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="n">
-        <v>7335.64453125</v>
+        <v>7048.53515625</v>
       </c>
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr"/>
@@ -3019,7 +3019,7 @@
       <c r="A64" t="inlineStr"/>
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="n">
-        <v>7622.75390625</v>
+        <v>7335.64453125</v>
       </c>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr"/>
@@ -3035,7 +3035,7 @@
       <c r="A65" t="inlineStr"/>
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="n">
-        <v>9072.65625</v>
+        <v>7622.75390625</v>
       </c>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr"/>
@@ -3050,10 +3050,10 @@
     <row r="66">
       <c r="A66" t="inlineStr"/>
       <c r="B66" t="inlineStr"/>
-      <c r="C66" t="inlineStr"/>
-      <c r="D66" t="n">
-        <v>645.99609375</v>
-      </c>
+      <c r="C66" t="n">
+        <v>9072.65625</v>
+      </c>
+      <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr"/>
@@ -3068,7 +3068,7 @@
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr"/>
       <c r="D67" t="n">
-        <v>746.484375</v>
+        <v>645.99609375</v>
       </c>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr"/>
@@ -3084,7 +3084,7 @@
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="n">
-        <v>861.328125</v>
+        <v>746.484375</v>
       </c>
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr"/>
@@ -3100,7 +3100,7 @@
       <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr"/>
       <c r="D69" t="n">
-        <v>990.52734375</v>
+        <v>861.328125</v>
       </c>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr"/>
@@ -3116,7 +3116,7 @@
       <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr"/>
       <c r="D70" t="n">
-        <v>1047.94921875</v>
+        <v>990.52734375</v>
       </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
@@ -3132,7 +3132,7 @@
       <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr"/>
       <c r="D71" t="n">
-        <v>1306.34765625</v>
+        <v>1047.94921875</v>
       </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr"/>
@@ -3148,7 +3148,7 @@
       <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr"/>
       <c r="D72" t="n">
-        <v>1478.61328125</v>
+        <v>1306.34765625</v>
       </c>
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr"/>
@@ -3164,7 +3164,7 @@
       <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr"/>
       <c r="D73" t="n">
-        <v>1550.390625</v>
+        <v>1478.61328125</v>
       </c>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr"/>
@@ -3180,7 +3180,7 @@
       <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr"/>
       <c r="D74" t="n">
-        <v>1622.16796875</v>
+        <v>1550.390625</v>
       </c>
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr"/>
@@ -3196,7 +3196,7 @@
       <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr"/>
       <c r="D75" t="n">
-        <v>1722.65625</v>
+        <v>1622.16796875</v>
       </c>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr"/>
@@ -3212,7 +3212,7 @@
       <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr"/>
       <c r="D76" t="n">
-        <v>1794.43359375</v>
+        <v>1722.65625</v>
       </c>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr"/>
@@ -3228,7 +3228,7 @@
       <c r="B77" t="inlineStr"/>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="n">
-        <v>1894.921875</v>
+        <v>1794.43359375</v>
       </c>
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr"/>
@@ -3244,7 +3244,7 @@
       <c r="B78" t="inlineStr"/>
       <c r="C78" t="inlineStr"/>
       <c r="D78" t="n">
-        <v>2024.12109375</v>
+        <v>1894.921875</v>
       </c>
       <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr"/>
@@ -3260,7 +3260,7 @@
       <c r="B79" t="inlineStr"/>
       <c r="C79" t="inlineStr"/>
       <c r="D79" t="n">
-        <v>2239.453125</v>
+        <v>2024.12109375</v>
       </c>
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr"/>
@@ -3276,7 +3276,7 @@
       <c r="B80" t="inlineStr"/>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
-        <v>2756.25</v>
+        <v>2239.453125</v>
       </c>
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr"/>
@@ -3292,7 +3292,7 @@
       <c r="B81" t="inlineStr"/>
       <c r="C81" t="inlineStr"/>
       <c r="D81" t="n">
-        <v>3043.359375</v>
+        <v>2756.25</v>
       </c>
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr"/>
@@ -3308,7 +3308,7 @@
       <c r="B82" t="inlineStr"/>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="n">
-        <v>3172.55859375</v>
+        <v>3043.359375</v>
       </c>
       <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr"/>
@@ -3324,7 +3324,7 @@
       <c r="B83" t="inlineStr"/>
       <c r="C83" t="inlineStr"/>
       <c r="D83" t="n">
-        <v>4005.17578125</v>
+        <v>3172.55859375</v>
       </c>
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr"/>
@@ -3340,7 +3340,7 @@
       <c r="B84" t="inlineStr"/>
       <c r="C84" t="inlineStr"/>
       <c r="D84" t="n">
-        <v>4177.44140625</v>
+        <v>4005.17578125</v>
       </c>
       <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr"/>
@@ -3355,10 +3355,10 @@
       <c r="A85" t="inlineStr"/>
       <c r="B85" t="inlineStr"/>
       <c r="C85" t="inlineStr"/>
-      <c r="D85" t="inlineStr"/>
-      <c r="E85" t="n">
-        <v>602.9296875</v>
-      </c>
+      <c r="D85" t="n">
+        <v>4177.44140625</v>
+      </c>
+      <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr"/>
@@ -3373,7 +3373,7 @@
       <c r="C86" t="inlineStr"/>
       <c r="D86" t="inlineStr"/>
       <c r="E86" t="n">
-        <v>732.12890625</v>
+        <v>602.9296875</v>
       </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr"/>
@@ -3389,7 +3389,7 @@
       <c r="C87" t="inlineStr"/>
       <c r="D87" t="inlineStr"/>
       <c r="E87" t="n">
-        <v>789.55078125</v>
+        <v>660.3515625</v>
       </c>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr"/>
@@ -3405,7 +3405,7 @@
       <c r="C88" t="inlineStr"/>
       <c r="D88" t="inlineStr"/>
       <c r="E88" t="n">
-        <v>846.97265625</v>
+        <v>732.12890625</v>
       </c>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr"/>
@@ -3421,7 +3421,7 @@
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="inlineStr"/>
       <c r="E89" t="n">
-        <v>904.39453125</v>
+        <v>789.55078125</v>
       </c>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
@@ -3437,7 +3437,7 @@
       <c r="C90" t="inlineStr"/>
       <c r="D90" t="inlineStr"/>
       <c r="E90" t="n">
-        <v>1234.5703125</v>
+        <v>846.97265625</v>
       </c>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr"/>
@@ -3453,7 +3453,7 @@
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="inlineStr"/>
       <c r="E91" t="n">
-        <v>1435.546875</v>
+        <v>904.39453125</v>
       </c>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr"/>
@@ -3469,7 +3469,7 @@
       <c r="C92" t="inlineStr"/>
       <c r="D92" t="inlineStr"/>
       <c r="E92" t="n">
-        <v>1708.30078125</v>
+        <v>1234.5703125</v>
       </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
@@ -3485,7 +3485,7 @@
       <c r="C93" t="inlineStr"/>
       <c r="D93" t="inlineStr"/>
       <c r="E93" t="n">
-        <v>1966.69921875</v>
+        <v>1435.546875</v>
       </c>
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr"/>
@@ -3501,7 +3501,7 @@
       <c r="C94" t="inlineStr"/>
       <c r="D94" t="inlineStr"/>
       <c r="E94" t="n">
-        <v>3560.15625</v>
+        <v>1708.30078125</v>
       </c>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr"/>
@@ -3517,7 +3517,7 @@
       <c r="C95" t="inlineStr"/>
       <c r="D95" t="inlineStr"/>
       <c r="E95" t="n">
-        <v>4062.59765625</v>
+        <v>1966.69921875</v>
       </c>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
@@ -3533,7 +3533,7 @@
       <c r="C96" t="inlineStr"/>
       <c r="D96" t="inlineStr"/>
       <c r="E96" t="n">
-        <v>4981.34765625</v>
+        <v>3560.15625</v>
       </c>
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr"/>
@@ -3549,7 +3549,7 @@
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="inlineStr"/>
       <c r="E97" t="n">
-        <v>7278.22265625</v>
+        <v>4062.59765625</v>
       </c>
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr"/>
@@ -3564,10 +3564,10 @@
       <c r="B98" t="inlineStr"/>
       <c r="C98" t="inlineStr"/>
       <c r="D98" t="inlineStr"/>
-      <c r="E98" t="inlineStr"/>
-      <c r="F98" t="n">
-        <v>1076.66015625</v>
-      </c>
+      <c r="E98" t="n">
+        <v>4981.34765625</v>
+      </c>
+      <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr"/>
       <c r="I98" t="inlineStr"/>
@@ -3580,10 +3580,10 @@
       <c r="B99" t="inlineStr"/>
       <c r="C99" t="inlineStr"/>
       <c r="D99" t="inlineStr"/>
-      <c r="E99" t="inlineStr"/>
-      <c r="F99" t="n">
-        <v>1119.7265625</v>
-      </c>
+      <c r="E99" t="n">
+        <v>7278.22265625</v>
+      </c>
+      <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr"/>
       <c r="H99" t="inlineStr"/>
       <c r="I99" t="inlineStr"/>
@@ -3598,7 +3598,7 @@
       <c r="D100" t="inlineStr"/>
       <c r="E100" t="inlineStr"/>
       <c r="F100" t="n">
-        <v>1291.9921875</v>
+        <v>1076.66015625</v>
       </c>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr"/>
@@ -3614,7 +3614,7 @@
       <c r="D101" t="inlineStr"/>
       <c r="E101" t="inlineStr"/>
       <c r="F101" t="n">
-        <v>1579.1015625</v>
+        <v>1119.7265625</v>
       </c>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="inlineStr"/>
@@ -3630,7 +3630,7 @@
       <c r="D102" t="inlineStr"/>
       <c r="E102" t="inlineStr"/>
       <c r="F102" t="n">
-        <v>1722.65625</v>
+        <v>1291.9921875</v>
       </c>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="inlineStr"/>
@@ -3646,7 +3646,7 @@
       <c r="D103" t="inlineStr"/>
       <c r="E103" t="inlineStr"/>
       <c r="F103" t="n">
-        <v>1837.5</v>
+        <v>1579.1015625</v>
       </c>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr"/>
@@ -3662,7 +3662,7 @@
       <c r="D104" t="inlineStr"/>
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="n">
-        <v>2339.94140625</v>
+        <v>1722.65625</v>
       </c>
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="inlineStr"/>
@@ -3678,7 +3678,7 @@
       <c r="D105" t="inlineStr"/>
       <c r="E105" t="inlineStr"/>
       <c r="F105" t="n">
-        <v>2813.671875</v>
+        <v>1837.5</v>
       </c>
       <c r="G105" t="inlineStr"/>
       <c r="H105" t="inlineStr"/>
@@ -3694,7 +3694,7 @@
       <c r="D106" t="inlineStr"/>
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="n">
-        <v>3072.0703125</v>
+        <v>2339.94140625</v>
       </c>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="inlineStr"/>
@@ -3710,7 +3710,7 @@
       <c r="D107" t="inlineStr"/>
       <c r="E107" t="inlineStr"/>
       <c r="F107" t="n">
-        <v>3402.24609375</v>
+        <v>2813.671875</v>
       </c>
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr"/>
@@ -3726,7 +3726,7 @@
       <c r="D108" t="inlineStr"/>
       <c r="E108" t="inlineStr"/>
       <c r="F108" t="n">
-        <v>4048.2421875</v>
+        <v>3072.0703125</v>
       </c>
       <c r="G108" t="inlineStr"/>
       <c r="H108" t="inlineStr"/>
@@ -3742,7 +3742,7 @@
       <c r="D109" t="inlineStr"/>
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="n">
-        <v>5124.90234375</v>
+        <v>3402.24609375</v>
       </c>
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr"/>
@@ -3758,7 +3758,7 @@
       <c r="D110" t="inlineStr"/>
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="n">
-        <v>5842.67578125</v>
+        <v>4048.2421875</v>
       </c>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr"/>
@@ -3774,7 +3774,7 @@
       <c r="D111" t="inlineStr"/>
       <c r="E111" t="inlineStr"/>
       <c r="F111" t="n">
-        <v>7938.57421875</v>
+        <v>5124.90234375</v>
       </c>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr"/>
@@ -3790,7 +3790,7 @@
       <c r="D112" t="inlineStr"/>
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="n">
-        <v>8311.81640625</v>
+        <v>5842.67578125</v>
       </c>
       <c r="G112" t="inlineStr"/>
       <c r="H112" t="inlineStr"/>
@@ -3806,7 +3806,7 @@
       <c r="D113" t="inlineStr"/>
       <c r="E113" t="inlineStr"/>
       <c r="F113" t="n">
-        <v>8670.703125</v>
+        <v>7938.57421875</v>
       </c>
       <c r="G113" t="inlineStr"/>
       <c r="H113" t="inlineStr"/>
@@ -3821,10 +3821,10 @@
       <c r="C114" t="inlineStr"/>
       <c r="D114" t="inlineStr"/>
       <c r="E114" t="inlineStr"/>
-      <c r="F114" t="inlineStr"/>
-      <c r="G114" t="n">
-        <v>545.5078125</v>
-      </c>
+      <c r="F114" t="n">
+        <v>8311.81640625</v>
+      </c>
+      <c r="G114" t="inlineStr"/>
       <c r="H114" t="inlineStr"/>
       <c r="I114" t="inlineStr"/>
       <c r="J114" t="inlineStr"/>
@@ -3837,10 +3837,10 @@
       <c r="C115" t="inlineStr"/>
       <c r="D115" t="inlineStr"/>
       <c r="E115" t="inlineStr"/>
-      <c r="F115" t="inlineStr"/>
-      <c r="G115" t="n">
-        <v>875.68359375</v>
-      </c>
+      <c r="F115" t="n">
+        <v>8670.703125</v>
+      </c>
+      <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr"/>
       <c r="I115" t="inlineStr"/>
       <c r="J115" t="inlineStr"/>
@@ -3855,7 +3855,7 @@
       <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="n">
-        <v>1220.21484375</v>
+        <v>545.5078125</v>
       </c>
       <c r="H116" t="inlineStr"/>
       <c r="I116" t="inlineStr"/>
@@ -3871,7 +3871,7 @@
       <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="n">
-        <v>1291.9921875</v>
+        <v>875.68359375</v>
       </c>
       <c r="H117" t="inlineStr"/>
       <c r="I117" t="inlineStr"/>
@@ -3887,7 +3887,7 @@
       <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="n">
-        <v>1349.4140625</v>
+        <v>1220.21484375</v>
       </c>
       <c r="H118" t="inlineStr"/>
       <c r="I118" t="inlineStr"/>
@@ -3903,7 +3903,7 @@
       <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr"/>
       <c r="G119" t="n">
-        <v>1492.96875</v>
+        <v>1291.9921875</v>
       </c>
       <c r="H119" t="inlineStr"/>
       <c r="I119" t="inlineStr"/>
@@ -3919,7 +3919,7 @@
       <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="n">
-        <v>1880.56640625</v>
+        <v>1349.4140625</v>
       </c>
       <c r="H120" t="inlineStr"/>
       <c r="I120" t="inlineStr"/>
@@ -3935,7 +3935,7 @@
       <c r="E121" t="inlineStr"/>
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="n">
-        <v>3043.359375</v>
+        <v>1492.96875</v>
       </c>
       <c r="H121" t="inlineStr"/>
       <c r="I121" t="inlineStr"/>
@@ -3951,7 +3951,7 @@
       <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="n">
-        <v>3158.203125</v>
+        <v>1880.56640625</v>
       </c>
       <c r="H122" t="inlineStr"/>
       <c r="I122" t="inlineStr"/>
@@ -3967,7 +3967,7 @@
       <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="n">
-        <v>3301.7578125</v>
+        <v>3043.359375</v>
       </c>
       <c r="H123" t="inlineStr"/>
       <c r="I123" t="inlineStr"/>
@@ -3983,7 +3983,7 @@
       <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="n">
-        <v>3789.84375</v>
+        <v>3158.203125</v>
       </c>
       <c r="H124" t="inlineStr"/>
       <c r="I124" t="inlineStr"/>
@@ -3998,10 +3998,10 @@
       <c r="D125" t="inlineStr"/>
       <c r="E125" t="inlineStr"/>
       <c r="F125" t="inlineStr"/>
-      <c r="G125" t="inlineStr"/>
-      <c r="H125" t="n">
-        <v>732.12890625</v>
-      </c>
+      <c r="G125" t="n">
+        <v>3301.7578125</v>
+      </c>
+      <c r="H125" t="inlineStr"/>
       <c r="I125" t="inlineStr"/>
       <c r="J125" t="inlineStr"/>
       <c r="K125" t="inlineStr"/>
@@ -4014,10 +4014,10 @@
       <c r="D126" t="inlineStr"/>
       <c r="E126" t="inlineStr"/>
       <c r="F126" t="inlineStr"/>
-      <c r="G126" t="inlineStr"/>
-      <c r="H126" t="n">
-        <v>990.52734375</v>
-      </c>
+      <c r="G126" t="n">
+        <v>3789.84375</v>
+      </c>
+      <c r="H126" t="inlineStr"/>
       <c r="I126" t="inlineStr"/>
       <c r="J126" t="inlineStr"/>
       <c r="K126" t="inlineStr"/>
@@ -4032,7 +4032,7 @@
       <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr"/>
       <c r="H127" t="n">
-        <v>1205.859375</v>
+        <v>732.12890625</v>
       </c>
       <c r="I127" t="inlineStr"/>
       <c r="J127" t="inlineStr"/>
@@ -4048,7 +4048,7 @@
       <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr"/>
       <c r="H128" t="n">
-        <v>1291.9921875</v>
+        <v>990.52734375</v>
       </c>
       <c r="I128" t="inlineStr"/>
       <c r="J128" t="inlineStr"/>
@@ -4064,7 +4064,7 @@
       <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="n">
-        <v>1636.5234375</v>
+        <v>1205.859375</v>
       </c>
       <c r="I129" t="inlineStr"/>
       <c r="J129" t="inlineStr"/>
@@ -4080,7 +4080,7 @@
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr"/>
       <c r="H130" t="n">
-        <v>2110.25390625</v>
+        <v>1291.9921875</v>
       </c>
       <c r="I130" t="inlineStr"/>
       <c r="J130" t="inlineStr"/>
@@ -4096,7 +4096,7 @@
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="n">
-        <v>2225.09765625</v>
+        <v>1636.5234375</v>
       </c>
       <c r="I131" t="inlineStr"/>
       <c r="J131" t="inlineStr"/>
@@ -4112,7 +4112,7 @@
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr"/>
       <c r="H132" t="n">
-        <v>3115.13671875</v>
+        <v>2110.25390625</v>
       </c>
       <c r="I132" t="inlineStr"/>
       <c r="J132" t="inlineStr"/>
@@ -4128,7 +4128,7 @@
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="n">
-        <v>4335.3515625</v>
+        <v>2225.09765625</v>
       </c>
       <c r="I133" t="inlineStr"/>
       <c r="J133" t="inlineStr"/>
@@ -4144,7 +4144,7 @@
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="n">
-        <v>5010.05859375</v>
+        <v>3115.13671875</v>
       </c>
       <c r="I134" t="inlineStr"/>
       <c r="J134" t="inlineStr"/>
@@ -4159,10 +4159,10 @@
       <c r="E135" t="inlineStr"/>
       <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr"/>
-      <c r="H135" t="inlineStr"/>
-      <c r="I135" t="n">
-        <v>703.41796875</v>
-      </c>
+      <c r="H135" t="n">
+        <v>4335.3515625</v>
+      </c>
+      <c r="I135" t="inlineStr"/>
       <c r="J135" t="inlineStr"/>
       <c r="K135" t="inlineStr"/>
       <c r="L135" t="inlineStr"/>
@@ -4175,10 +4175,10 @@
       <c r="E136" t="inlineStr"/>
       <c r="F136" t="inlineStr"/>
       <c r="G136" t="inlineStr"/>
-      <c r="H136" t="inlineStr"/>
-      <c r="I136" t="n">
-        <v>990.52734375</v>
-      </c>
+      <c r="H136" t="n">
+        <v>5010.05859375</v>
+      </c>
+      <c r="I136" t="inlineStr"/>
       <c r="J136" t="inlineStr"/>
       <c r="K136" t="inlineStr"/>
       <c r="L136" t="inlineStr"/>
@@ -4193,7 +4193,7 @@
       <c r="G137" t="inlineStr"/>
       <c r="H137" t="inlineStr"/>
       <c r="I137" t="n">
-        <v>1679.58984375</v>
+        <v>703.41796875</v>
       </c>
       <c r="J137" t="inlineStr"/>
       <c r="K137" t="inlineStr"/>
@@ -4209,7 +4209,7 @@
       <c r="G138" t="inlineStr"/>
       <c r="H138" t="inlineStr"/>
       <c r="I138" t="n">
-        <v>1780.078125</v>
+        <v>990.52734375</v>
       </c>
       <c r="J138" t="inlineStr"/>
       <c r="K138" t="inlineStr"/>
@@ -4225,7 +4225,7 @@
       <c r="G139" t="inlineStr"/>
       <c r="H139" t="inlineStr"/>
       <c r="I139" t="n">
-        <v>1894.921875</v>
+        <v>1492.96875</v>
       </c>
       <c r="J139" t="inlineStr"/>
       <c r="K139" t="inlineStr"/>
@@ -4241,7 +4241,7 @@
       <c r="G140" t="inlineStr"/>
       <c r="H140" t="inlineStr"/>
       <c r="I140" t="n">
-        <v>2138.96484375</v>
+        <v>1679.58984375</v>
       </c>
       <c r="J140" t="inlineStr"/>
       <c r="K140" t="inlineStr"/>
@@ -4257,7 +4257,7 @@
       <c r="G141" t="inlineStr"/>
       <c r="H141" t="inlineStr"/>
       <c r="I141" t="n">
-        <v>3258.69140625</v>
+        <v>1780.078125</v>
       </c>
       <c r="J141" t="inlineStr"/>
       <c r="K141" t="inlineStr"/>
@@ -4273,7 +4273,7 @@
       <c r="G142" t="inlineStr"/>
       <c r="H142" t="inlineStr"/>
       <c r="I142" t="n">
-        <v>3732.421875</v>
+        <v>1894.921875</v>
       </c>
       <c r="J142" t="inlineStr"/>
       <c r="K142" t="inlineStr"/>
@@ -4289,7 +4289,7 @@
       <c r="G143" t="inlineStr"/>
       <c r="H143" t="inlineStr"/>
       <c r="I143" t="n">
-        <v>4163.0859375</v>
+        <v>2138.96484375</v>
       </c>
       <c r="J143" t="inlineStr"/>
       <c r="K143" t="inlineStr"/>
@@ -4305,7 +4305,7 @@
       <c r="G144" t="inlineStr"/>
       <c r="H144" t="inlineStr"/>
       <c r="I144" t="n">
-        <v>4407.12890625</v>
+        <v>3258.69140625</v>
       </c>
       <c r="J144" t="inlineStr"/>
       <c r="K144" t="inlineStr"/>
@@ -4321,7 +4321,7 @@
       <c r="G145" t="inlineStr"/>
       <c r="H145" t="inlineStr"/>
       <c r="I145" t="n">
-        <v>5555.56640625</v>
+        <v>3732.421875</v>
       </c>
       <c r="J145" t="inlineStr"/>
       <c r="K145" t="inlineStr"/>
@@ -4337,7 +4337,7 @@
       <c r="G146" t="inlineStr"/>
       <c r="H146" t="inlineStr"/>
       <c r="I146" t="n">
-        <v>6474.31640625</v>
+        <v>4163.0859375</v>
       </c>
       <c r="J146" t="inlineStr"/>
       <c r="K146" t="inlineStr"/>
@@ -4353,7 +4353,7 @@
       <c r="G147" t="inlineStr"/>
       <c r="H147" t="inlineStr"/>
       <c r="I147" t="n">
-        <v>7665.8203125</v>
+        <v>4407.12890625</v>
       </c>
       <c r="J147" t="inlineStr"/>
       <c r="K147" t="inlineStr"/>
@@ -4369,7 +4369,7 @@
       <c r="G148" t="inlineStr"/>
       <c r="H148" t="inlineStr"/>
       <c r="I148" t="n">
-        <v>9115.72265625</v>
+        <v>5254.1015625</v>
       </c>
       <c r="J148" t="inlineStr"/>
       <c r="K148" t="inlineStr"/>
@@ -4385,7 +4385,7 @@
       <c r="G149" t="inlineStr"/>
       <c r="H149" t="inlineStr"/>
       <c r="I149" t="n">
-        <v>11714.0625</v>
+        <v>5555.56640625</v>
       </c>
       <c r="J149" t="inlineStr"/>
       <c r="K149" t="inlineStr"/>
@@ -4400,10 +4400,10 @@
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr"/>
       <c r="H150" t="inlineStr"/>
-      <c r="I150" t="inlineStr"/>
-      <c r="J150" t="n">
-        <v>660.3515625</v>
-      </c>
+      <c r="I150" t="n">
+        <v>6474.31640625</v>
+      </c>
+      <c r="J150" t="inlineStr"/>
       <c r="K150" t="inlineStr"/>
       <c r="L150" t="inlineStr"/>
     </row>
@@ -4416,10 +4416,10 @@
       <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr"/>
       <c r="H151" t="inlineStr"/>
-      <c r="I151" t="inlineStr"/>
-      <c r="J151" t="n">
-        <v>904.39453125</v>
-      </c>
+      <c r="I151" t="n">
+        <v>7665.8203125</v>
+      </c>
+      <c r="J151" t="inlineStr"/>
       <c r="K151" t="inlineStr"/>
       <c r="L151" t="inlineStr"/>
     </row>
@@ -4432,10 +4432,10 @@
       <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr"/>
       <c r="H152" t="inlineStr"/>
-      <c r="I152" t="inlineStr"/>
-      <c r="J152" t="n">
-        <v>976.171875</v>
-      </c>
+      <c r="I152" t="n">
+        <v>9115.72265625</v>
+      </c>
+      <c r="J152" t="inlineStr"/>
       <c r="K152" t="inlineStr"/>
       <c r="L152" t="inlineStr"/>
     </row>
@@ -4448,10 +4448,10 @@
       <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr"/>
       <c r="H153" t="inlineStr"/>
-      <c r="I153" t="inlineStr"/>
-      <c r="J153" t="n">
-        <v>1277.63671875</v>
-      </c>
+      <c r="I153" t="n">
+        <v>11714.0625</v>
+      </c>
+      <c r="J153" t="inlineStr"/>
       <c r="K153" t="inlineStr"/>
       <c r="L153" t="inlineStr"/>
     </row>
@@ -4466,7 +4466,7 @@
       <c r="H154" t="inlineStr"/>
       <c r="I154" t="inlineStr"/>
       <c r="J154" t="n">
-        <v>1335.05859375</v>
+        <v>660.3515625</v>
       </c>
       <c r="K154" t="inlineStr"/>
       <c r="L154" t="inlineStr"/>
@@ -4482,7 +4482,7 @@
       <c r="H155" t="inlineStr"/>
       <c r="I155" t="inlineStr"/>
       <c r="J155" t="n">
-        <v>1435.546875</v>
+        <v>904.39453125</v>
       </c>
       <c r="K155" t="inlineStr"/>
       <c r="L155" t="inlineStr"/>
@@ -4498,7 +4498,7 @@
       <c r="H156" t="inlineStr"/>
       <c r="I156" t="inlineStr"/>
       <c r="J156" t="n">
-        <v>1521.6796875</v>
+        <v>976.171875</v>
       </c>
       <c r="K156" t="inlineStr"/>
       <c r="L156" t="inlineStr"/>
@@ -4514,7 +4514,7 @@
       <c r="H157" t="inlineStr"/>
       <c r="I157" t="inlineStr"/>
       <c r="J157" t="n">
-        <v>1665.234375</v>
+        <v>1277.63671875</v>
       </c>
       <c r="K157" t="inlineStr"/>
       <c r="L157" t="inlineStr"/>
@@ -4530,7 +4530,7 @@
       <c r="H158" t="inlineStr"/>
       <c r="I158" t="inlineStr"/>
       <c r="J158" t="n">
-        <v>1808.7890625</v>
+        <v>1335.05859375</v>
       </c>
       <c r="K158" t="inlineStr"/>
       <c r="L158" t="inlineStr"/>
@@ -4546,7 +4546,7 @@
       <c r="H159" t="inlineStr"/>
       <c r="I159" t="inlineStr"/>
       <c r="J159" t="n">
-        <v>1923.6328125</v>
+        <v>1435.546875</v>
       </c>
       <c r="K159" t="inlineStr"/>
       <c r="L159" t="inlineStr"/>
@@ -4562,7 +4562,7 @@
       <c r="H160" t="inlineStr"/>
       <c r="I160" t="inlineStr"/>
       <c r="J160" t="n">
-        <v>2038.4765625</v>
+        <v>1521.6796875</v>
       </c>
       <c r="K160" t="inlineStr"/>
       <c r="L160" t="inlineStr"/>
@@ -4578,7 +4578,7 @@
       <c r="H161" t="inlineStr"/>
       <c r="I161" t="inlineStr"/>
       <c r="J161" t="n">
-        <v>2153.3203125</v>
+        <v>1665.234375</v>
       </c>
       <c r="K161" t="inlineStr"/>
       <c r="L161" t="inlineStr"/>
@@ -4594,7 +4594,7 @@
       <c r="H162" t="inlineStr"/>
       <c r="I162" t="inlineStr"/>
       <c r="J162" t="n">
-        <v>2282.51953125</v>
+        <v>1808.7890625</v>
       </c>
       <c r="K162" t="inlineStr"/>
       <c r="L162" t="inlineStr"/>
@@ -4610,7 +4610,7 @@
       <c r="H163" t="inlineStr"/>
       <c r="I163" t="inlineStr"/>
       <c r="J163" t="n">
-        <v>2698.828125</v>
+        <v>1923.6328125</v>
       </c>
       <c r="K163" t="inlineStr"/>
       <c r="L163" t="inlineStr"/>
@@ -4626,7 +4626,7 @@
       <c r="H164" t="inlineStr"/>
       <c r="I164" t="inlineStr"/>
       <c r="J164" t="n">
-        <v>2842.3828125</v>
+        <v>2038.4765625</v>
       </c>
       <c r="K164" t="inlineStr"/>
       <c r="L164" t="inlineStr"/>
@@ -4642,7 +4642,7 @@
       <c r="H165" t="inlineStr"/>
       <c r="I165" t="inlineStr"/>
       <c r="J165" t="n">
-        <v>3631.93359375</v>
+        <v>2153.3203125</v>
       </c>
       <c r="K165" t="inlineStr"/>
       <c r="L165" t="inlineStr"/>
@@ -4658,7 +4658,7 @@
       <c r="H166" t="inlineStr"/>
       <c r="I166" t="inlineStr"/>
       <c r="J166" t="n">
-        <v>6043.65234375</v>
+        <v>2282.51953125</v>
       </c>
       <c r="K166" t="inlineStr"/>
       <c r="L166" t="inlineStr"/>
@@ -4674,7 +4674,7 @@
       <c r="H167" t="inlineStr"/>
       <c r="I167" t="inlineStr"/>
       <c r="J167" t="n">
-        <v>7278.22265625</v>
+        <v>2698.828125</v>
       </c>
       <c r="K167" t="inlineStr"/>
       <c r="L167" t="inlineStr"/>
@@ -4689,10 +4689,10 @@
       <c r="G168" t="inlineStr"/>
       <c r="H168" t="inlineStr"/>
       <c r="I168" t="inlineStr"/>
-      <c r="J168" t="inlineStr"/>
-      <c r="K168" t="n">
-        <v>602.9296875</v>
-      </c>
+      <c r="J168" t="n">
+        <v>2842.3828125</v>
+      </c>
+      <c r="K168" t="inlineStr"/>
       <c r="L168" t="inlineStr"/>
     </row>
     <row r="169">
@@ -4705,10 +4705,10 @@
       <c r="G169" t="inlineStr"/>
       <c r="H169" t="inlineStr"/>
       <c r="I169" t="inlineStr"/>
-      <c r="J169" t="inlineStr"/>
-      <c r="K169" t="n">
-        <v>861.328125</v>
-      </c>
+      <c r="J169" t="n">
+        <v>3631.93359375</v>
+      </c>
+      <c r="K169" t="inlineStr"/>
       <c r="L169" t="inlineStr"/>
     </row>
     <row r="170">
@@ -4721,10 +4721,10 @@
       <c r="G170" t="inlineStr"/>
       <c r="H170" t="inlineStr"/>
       <c r="I170" t="inlineStr"/>
-      <c r="J170" t="inlineStr"/>
-      <c r="K170" t="n">
-        <v>933.10546875</v>
-      </c>
+      <c r="J170" t="n">
+        <v>6043.65234375</v>
+      </c>
+      <c r="K170" t="inlineStr"/>
       <c r="L170" t="inlineStr"/>
     </row>
     <row r="171">
@@ -4737,10 +4737,10 @@
       <c r="G171" t="inlineStr"/>
       <c r="H171" t="inlineStr"/>
       <c r="I171" t="inlineStr"/>
-      <c r="J171" t="inlineStr"/>
-      <c r="K171" t="n">
-        <v>1263.28125</v>
-      </c>
+      <c r="J171" t="n">
+        <v>7278.22265625</v>
+      </c>
+      <c r="K171" t="inlineStr"/>
       <c r="L171" t="inlineStr"/>
     </row>
     <row r="172">
@@ -4755,7 +4755,7 @@
       <c r="I172" t="inlineStr"/>
       <c r="J172" t="inlineStr"/>
       <c r="K172" t="n">
-        <v>1349.4140625</v>
+        <v>602.9296875</v>
       </c>
       <c r="L172" t="inlineStr"/>
     </row>
@@ -4771,7 +4771,7 @@
       <c r="I173" t="inlineStr"/>
       <c r="J173" t="inlineStr"/>
       <c r="K173" t="n">
-        <v>1536.03515625</v>
+        <v>861.328125</v>
       </c>
       <c r="L173" t="inlineStr"/>
     </row>
@@ -4787,7 +4787,7 @@
       <c r="I174" t="inlineStr"/>
       <c r="J174" t="inlineStr"/>
       <c r="K174" t="n">
-        <v>1622.16796875</v>
+        <v>933.10546875</v>
       </c>
       <c r="L174" t="inlineStr"/>
     </row>
@@ -4803,7 +4803,7 @@
       <c r="I175" t="inlineStr"/>
       <c r="J175" t="inlineStr"/>
       <c r="K175" t="n">
-        <v>2253.80859375</v>
+        <v>1263.28125</v>
       </c>
       <c r="L175" t="inlineStr"/>
     </row>
@@ -4819,7 +4819,7 @@
       <c r="I176" t="inlineStr"/>
       <c r="J176" t="inlineStr"/>
       <c r="K176" t="n">
-        <v>2828.02734375</v>
+        <v>1349.4140625</v>
       </c>
       <c r="L176" t="inlineStr"/>
     </row>
@@ -4835,7 +4835,7 @@
       <c r="I177" t="inlineStr"/>
       <c r="J177" t="inlineStr"/>
       <c r="K177" t="n">
-        <v>3086.42578125</v>
+        <v>1536.03515625</v>
       </c>
       <c r="L177" t="inlineStr"/>
     </row>
@@ -4851,7 +4851,7 @@
       <c r="I178" t="inlineStr"/>
       <c r="J178" t="inlineStr"/>
       <c r="K178" t="n">
-        <v>3445.3125</v>
+        <v>1622.16796875</v>
       </c>
       <c r="L178" t="inlineStr"/>
     </row>
@@ -4867,7 +4867,7 @@
       <c r="I179" t="inlineStr"/>
       <c r="J179" t="inlineStr"/>
       <c r="K179" t="n">
-        <v>4378.41796875</v>
+        <v>2253.80859375</v>
       </c>
       <c r="L179" t="inlineStr"/>
     </row>
@@ -4883,7 +4883,7 @@
       <c r="I180" t="inlineStr"/>
       <c r="J180" t="inlineStr"/>
       <c r="K180" t="n">
-        <v>4521.97265625</v>
+        <v>2828.02734375</v>
       </c>
       <c r="L180" t="inlineStr"/>
     </row>
@@ -4899,7 +4899,7 @@
       <c r="I181" t="inlineStr"/>
       <c r="J181" t="inlineStr"/>
       <c r="K181" t="n">
-        <v>4722.94921875</v>
+        <v>3086.42578125</v>
       </c>
       <c r="L181" t="inlineStr"/>
     </row>
@@ -4915,7 +4915,7 @@
       <c r="I182" t="inlineStr"/>
       <c r="J182" t="inlineStr"/>
       <c r="K182" t="n">
-        <v>6058.0078125</v>
+        <v>3445.3125</v>
       </c>
       <c r="L182" t="inlineStr"/>
     </row>
@@ -4931,7 +4931,7 @@
       <c r="I183" t="inlineStr"/>
       <c r="J183" t="inlineStr"/>
       <c r="K183" t="n">
-        <v>6316.40625</v>
+        <v>4378.41796875</v>
       </c>
       <c r="L183" t="inlineStr"/>
     </row>
@@ -4946,10 +4946,10 @@
       <c r="H184" t="inlineStr"/>
       <c r="I184" t="inlineStr"/>
       <c r="J184" t="inlineStr"/>
-      <c r="K184" t="inlineStr"/>
-      <c r="L184" t="n">
-        <v>1406.8359375</v>
-      </c>
+      <c r="K184" t="n">
+        <v>4521.97265625</v>
+      </c>
+      <c r="L184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr"/>
@@ -4962,10 +4962,10 @@
       <c r="H185" t="inlineStr"/>
       <c r="I185" t="inlineStr"/>
       <c r="J185" t="inlineStr"/>
-      <c r="K185" t="inlineStr"/>
-      <c r="L185" t="n">
-        <v>1507.32421875</v>
-      </c>
+      <c r="K185" t="n">
+        <v>4722.94921875</v>
+      </c>
+      <c r="L185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr"/>
@@ -4978,10 +4978,10 @@
       <c r="H186" t="inlineStr"/>
       <c r="I186" t="inlineStr"/>
       <c r="J186" t="inlineStr"/>
-      <c r="K186" t="inlineStr"/>
-      <c r="L186" t="n">
-        <v>1622.16796875</v>
-      </c>
+      <c r="K186" t="n">
+        <v>6058.0078125</v>
+      </c>
+      <c r="L186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr"/>
@@ -4994,10 +4994,10 @@
       <c r="H187" t="inlineStr"/>
       <c r="I187" t="inlineStr"/>
       <c r="J187" t="inlineStr"/>
-      <c r="K187" t="inlineStr"/>
-      <c r="L187" t="n">
-        <v>1722.65625</v>
-      </c>
+      <c r="K187" t="n">
+        <v>6316.40625</v>
+      </c>
+      <c r="L187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr"/>
@@ -5012,7 +5012,7 @@
       <c r="J188" t="inlineStr"/>
       <c r="K188" t="inlineStr"/>
       <c r="L188" t="n">
-        <v>1880.56640625</v>
+        <v>1406.8359375</v>
       </c>
     </row>
     <row r="189">
@@ -5028,7 +5028,7 @@
       <c r="J189" t="inlineStr"/>
       <c r="K189" t="inlineStr"/>
       <c r="L189" t="n">
-        <v>2009.765625</v>
+        <v>1507.32421875</v>
       </c>
     </row>
     <row r="190">
@@ -5044,7 +5044,7 @@
       <c r="J190" t="inlineStr"/>
       <c r="K190" t="inlineStr"/>
       <c r="L190" t="n">
-        <v>2138.96484375</v>
+        <v>1622.16796875</v>
       </c>
     </row>
     <row r="191">
@@ -5060,7 +5060,7 @@
       <c r="J191" t="inlineStr"/>
       <c r="K191" t="inlineStr"/>
       <c r="L191" t="n">
-        <v>2296.875</v>
+        <v>1722.65625</v>
       </c>
     </row>
     <row r="192">
@@ -5076,7 +5076,7 @@
       <c r="J192" t="inlineStr"/>
       <c r="K192" t="inlineStr"/>
       <c r="L192" t="n">
-        <v>2469.140625</v>
+        <v>1880.56640625</v>
       </c>
     </row>
     <row r="193">
@@ -5092,7 +5092,7 @@
       <c r="J193" t="inlineStr"/>
       <c r="K193" t="inlineStr"/>
       <c r="L193" t="n">
-        <v>2612.6953125</v>
+        <v>2009.765625</v>
       </c>
     </row>
     <row r="194">
@@ -5108,7 +5108,7 @@
       <c r="J194" t="inlineStr"/>
       <c r="K194" t="inlineStr"/>
       <c r="L194" t="n">
-        <v>2756.25</v>
+        <v>2138.96484375</v>
       </c>
     </row>
     <row r="195">
@@ -5124,7 +5124,7 @@
       <c r="J195" t="inlineStr"/>
       <c r="K195" t="inlineStr"/>
       <c r="L195" t="n">
-        <v>2914.16015625</v>
+        <v>2296.875</v>
       </c>
     </row>
     <row r="196">
@@ -5140,7 +5140,7 @@
       <c r="J196" t="inlineStr"/>
       <c r="K196" t="inlineStr"/>
       <c r="L196" t="n">
-        <v>3072.0703125</v>
+        <v>2469.140625</v>
       </c>
     </row>
     <row r="197">
@@ -5156,7 +5156,7 @@
       <c r="J197" t="inlineStr"/>
       <c r="K197" t="inlineStr"/>
       <c r="L197" t="n">
-        <v>3273.046875</v>
+        <v>2612.6953125</v>
       </c>
     </row>
     <row r="198">
@@ -5172,6 +5172,70 @@
       <c r="J198" t="inlineStr"/>
       <c r="K198" t="inlineStr"/>
       <c r="L198" t="n">
+        <v>2756.25</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr"/>
+      <c r="B199" t="inlineStr"/>
+      <c r="C199" t="inlineStr"/>
+      <c r="D199" t="inlineStr"/>
+      <c r="E199" t="inlineStr"/>
+      <c r="F199" t="inlineStr"/>
+      <c r="G199" t="inlineStr"/>
+      <c r="H199" t="inlineStr"/>
+      <c r="I199" t="inlineStr"/>
+      <c r="J199" t="inlineStr"/>
+      <c r="K199" t="inlineStr"/>
+      <c r="L199" t="n">
+        <v>2914.16015625</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr"/>
+      <c r="B200" t="inlineStr"/>
+      <c r="C200" t="inlineStr"/>
+      <c r="D200" t="inlineStr"/>
+      <c r="E200" t="inlineStr"/>
+      <c r="F200" t="inlineStr"/>
+      <c r="G200" t="inlineStr"/>
+      <c r="H200" t="inlineStr"/>
+      <c r="I200" t="inlineStr"/>
+      <c r="J200" t="inlineStr"/>
+      <c r="K200" t="inlineStr"/>
+      <c r="L200" t="n">
+        <v>3072.0703125</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr"/>
+      <c r="B201" t="inlineStr"/>
+      <c r="C201" t="inlineStr"/>
+      <c r="D201" t="inlineStr"/>
+      <c r="E201" t="inlineStr"/>
+      <c r="F201" t="inlineStr"/>
+      <c r="G201" t="inlineStr"/>
+      <c r="H201" t="inlineStr"/>
+      <c r="I201" t="inlineStr"/>
+      <c r="J201" t="inlineStr"/>
+      <c r="K201" t="inlineStr"/>
+      <c r="L201" t="n">
+        <v>3273.046875</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr"/>
+      <c r="B202" t="inlineStr"/>
+      <c r="C202" t="inlineStr"/>
+      <c r="D202" t="inlineStr"/>
+      <c r="E202" t="inlineStr"/>
+      <c r="F202" t="inlineStr"/>
+      <c r="G202" t="inlineStr"/>
+      <c r="H202" t="inlineStr"/>
+      <c r="I202" t="inlineStr"/>
+      <c r="J202" t="inlineStr"/>
+      <c r="K202" t="inlineStr"/>
+      <c r="L202" t="n">
         <v>4134.375</v>
       </c>
     </row>

</xml_diff>